<commit_message>
Add Tencent, Zhipu, DeepSeek and xAI with archived vendor reports
</commit_message>
<xml_diff>
--- a/web/public/downloads/audit-2026-10-18.xlsx
+++ b/web/public/downloads/audit-2026-10-18.xlsx
@@ -18,6 +18,8 @@
     <sheet name="修订记录" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="访问日志" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="成绩补录审计" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="新增厂商模型" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="新增厂商证据文件" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$4:$B$19</definedName>
@@ -40,7 +42,9 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'修订记录'!$1:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'访问日志'!$A$4:$H$108</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'访问日志'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'成绩补录审计'!$A$4:$K$237</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'成绩补录审计'!$A$4:$K$272</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'新增厂商模型'!$A$1:$J$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'新增厂商证据文件'!$A$1:$F$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -141,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -170,6 +174,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -741,7 +748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -976,6 +983,18 @@
       <c r="B21" t="inlineStr">
         <is>
           <t>原2026-10-17工作簿完整保留在仓库snapshots/2026-10-17.xlsx。本文件为附加成绩证据后的导出版本。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>厂商扩展</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>新增腾讯、智谱GLM、DeepSeek、xAI共25个模型／版本、35条记录；网页和图片以章节／表格定位，不伪造PDF页码。所有记录见成绩补录审计表，新增模型和证据文件另列。</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K237"/>
+  <dimension ref="A1:K272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5270,7 +5289,7 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>PDF成绩补录审计 | 2026-10-18</t>
+          <t>公开报告成绩复核 | 2026-10-18</t>
         </is>
       </c>
       <c r="B1" s="10" t="n"/>
@@ -5287,7 +5306,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>复核196条已确认记录；原成绩43条，现已核实数值156条，新增数值113条。</t>
+          <t>复核218条已确认记录；原成绩43条，现已核实数值178条，新增数值135条。</t>
         </is>
       </c>
       <c r="B2" s="10" t="n"/>
@@ -17269,8 +17288,4219 @@
         </is>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0234</t>
+        </is>
+      </c>
+      <c r="B238" s="10" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Flash</t>
+        </is>
+      </c>
+      <c r="C238" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D238" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E238" s="10" t="inlineStr">
+        <is>
+          <t>76.7%</t>
+        </is>
+      </c>
+      <c r="F238" s="10" t="inlineStr"/>
+      <c r="G238" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H238" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-release-1.html 2026-07-31</t>
+        </is>
+      </c>
+      <c r="I238" s="10" t="inlineStr">
+        <is>
+          <t>Cybergym: 76.7</t>
+        </is>
+      </c>
+      <c r="J238" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 76.7, "unit": "percent", "configuration": "正式版Flash-0731；7月31日更新记录；DeepSeek Harness minimal，max effort，top_p=0.95，temperature=1.0；正式版专属成绩；本条模型日期使用正式版上线日。"}]</t>
+        </is>
+      </c>
+      <c r="K238" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0235</t>
+        </is>
+      </c>
+      <c r="B239" s="10" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Pro</t>
+        </is>
+      </c>
+      <c r="C239" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D239" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E239" s="10" t="inlineStr">
+        <is>
+          <t>83.3%</t>
+        </is>
+      </c>
+      <c r="F239" s="10" t="inlineStr"/>
+      <c r="G239" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H239" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-release-1.html 2026-08-13</t>
+        </is>
+      </c>
+      <c r="I239" s="10" t="inlineStr">
+        <is>
+          <t>Cybergym: 83.3</t>
+        </is>
+      </c>
+      <c r="J239" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 83.3, "unit": "percent", "configuration": "8月13日正式版；不可混作4月Preview成绩；正式版专属成绩；本条模型日期使用正式版上线日。"}]</t>
+        </is>
+      </c>
+      <c r="K239" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0236</t>
+        </is>
+      </c>
+      <c r="B240" s="10" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Flash-Vision-Exp</t>
+        </is>
+      </c>
+      <c r="C240" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D240" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E240" s="10" t="inlineStr">
+        <is>
+          <t>75.3%</t>
+        </is>
+      </c>
+      <c r="F240" s="10" t="inlineStr"/>
+      <c r="G240" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H240" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-vision-exp.html 基准表图片，CyberGym行；sources/vendors/DeepSeek/v4_260821_benchmark_en.png CyberGym行／Vision-Exp独立列</t>
+        </is>
+      </c>
+      <c r="I240" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym row: DeepSeek V4-Flash-Vision-Exp 75.3; DeepSeek V4-Flash-0731 76.7.
+CyberGym row: DeepSeek V4-Flash-Vision-Exp 75.3; DeepSeek V4-Flash-0731 76.7.</t>
+        </is>
+      </c>
+      <c r="J240" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 75.3, "unit": "percent", "configuration": "发布页图片Text-Based Agent Evaluation；DeepSeek Harness Minimal Mode；top_p=.95，temperature=1；模型独立列"}]</t>
+        </is>
+      </c>
+      <c r="K240" s="10" t="inlineStr">
+        <is>
+          <t>已人工读取官方基准表图片；原文goal.txt漏列。；原始图表：docs/DeepSeek/v4_260821_benchmark_en.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0237</t>
+        </is>
+      </c>
+      <c r="B241" s="10" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4.1-Flash</t>
+        </is>
+      </c>
+      <c r="C241" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D241" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E241" s="10" t="inlineStr">
+        <is>
+          <t>88.1%</t>
+        </is>
+      </c>
+      <c r="F241" s="10" t="inlineStr"/>
+      <c r="G241" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H241" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-release-1.html 2026-09-10；sources/vendors/DeepSeek/deepseek-v4-1-flash.pdf p.32-33</t>
+        </is>
+      </c>
+      <c r="I241" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym (Pass@1) 88.1
+CyberGym (Pass@1) 88.1</t>
+        </is>
+      </c>
+      <c r="J241" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 88.1, "unit": "percent", "configuration": "2026-09-10发布快照；官方日志原值；具体设置见技术报告"}]</t>
+        </is>
+      </c>
+      <c r="K241" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0238</t>
+        </is>
+      </c>
+      <c r="B242" s="10" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4.1-Flash</t>
+        </is>
+      </c>
+      <c r="C242" s="10" t="inlineStr">
+        <is>
+          <t>SEC-Bench Pro</t>
+        </is>
+      </c>
+      <c r="D242" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E242" s="10" t="inlineStr">
+        <is>
+          <t>62.8%</t>
+        </is>
+      </c>
+      <c r="F242" s="10" t="inlineStr"/>
+      <c r="G242" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H242" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-release-1.html 2026-09-10；sources/vendors/DeepSeek/deepseek-v4-1-flash.pdf p.32-33</t>
+        </is>
+      </c>
+      <c r="I242" s="10" t="inlineStr">
+        <is>
+          <t>SEC-Bench Pro (Pass@1) 62.8
+SEC-Bench Pro (Pass@1) 62.8</t>
+        </is>
+      </c>
+      <c r="J242" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "pass@1", "value": 62.8, "unit": "percent", "configuration": "2026-09-10发布快照；官方日志原值；具体设置见技术报告"}]</t>
+        </is>
+      </c>
+      <c r="K242" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0239</t>
+        </is>
+      </c>
+      <c r="B243" s="10" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4.1-Flash</t>
+        </is>
+      </c>
+      <c r="C243" s="10" t="inlineStr">
+        <is>
+          <t>ExploitGym</t>
+        </is>
+      </c>
+      <c r="D243" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E243" s="10" t="inlineStr">
+        <is>
+          <t>15.3%</t>
+        </is>
+      </c>
+      <c r="F243" s="10" t="inlineStr"/>
+      <c r="G243" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H243" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-release-1.html 2026-09-10；sources/vendors/DeepSeek/deepseek-v4-1-flash.pdf p.32-33</t>
+        </is>
+      </c>
+      <c r="I243" s="10" t="inlineStr">
+        <is>
+          <t>ExploitGym (Pass@1) 15.3
+ExploitGym (Pass@1) 15.3</t>
+        </is>
+      </c>
+      <c r="J243" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "pass@1", "value": 15.3, "unit": "percent", "configuration": "2026-09-10发布快照；官方日志原值；具体设置见技术报告"}]</t>
+        </is>
+      </c>
+      <c r="K243" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0240</t>
+        </is>
+      </c>
+      <c r="B244" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5</t>
+        </is>
+      </c>
+      <c r="C244" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D244" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E244" s="10" t="inlineStr">
+        <is>
+          <t>43.2%</t>
+        </is>
+      </c>
+      <c r="F244" s="10" t="inlineStr"/>
+      <c r="G244" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H244" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-release-1.mhtml Performance / Footnotes</t>
+        </is>
+      </c>
+      <c r="I244" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym 43.2 (GLM-5 column)</t>
+        </is>
+      </c>
+      <c r="J244" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 43.2, "unit": "percent", "configuration": "首发博客；Claude Code2.1.18，think，无web；1507任务，单次pass@1，250min/任务"}]</t>
+        </is>
+      </c>
+      <c r="K244" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0241</t>
+        </is>
+      </c>
+      <c r="B245" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5</t>
+        </is>
+      </c>
+      <c r="C245" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D245" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E245" s="10" t="inlineStr">
+        <is>
+          <t>48.3%</t>
+        </is>
+      </c>
+      <c r="F245" s="10" t="inlineStr"/>
+      <c r="G245" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H245" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-1.mhtml Performance table</t>
+        </is>
+      </c>
+      <c r="I245" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym 48.3 (GLM-5 comparison column)</t>
+        </is>
+      </c>
+      <c r="J245" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 48.3, "unit": "percent", "configuration": "后续GLM-5.1官方博客中的GLM-5比较列"}]</t>
+        </is>
+      </c>
+      <c r="K245" s="10" t="inlineStr">
+        <is>
+          <t>后续报告比较值；保留首发43.2，不覆盖原值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0242</t>
+        </is>
+      </c>
+      <c r="B246" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5.1</t>
+        </is>
+      </c>
+      <c r="C246" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D246" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E246" s="10" t="inlineStr">
+        <is>
+          <t>68.7%</t>
+        </is>
+      </c>
+      <c r="F246" s="10" t="inlineStr"/>
+      <c r="G246" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H246" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-1.mhtml Performance / Footnotes</t>
+        </is>
+      </c>
+      <c r="I246" s="10" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J246" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 68.7, "unit": "percent", "configuration": "Claude Code2.1.56，think，无web，temperature1，top_p1，max_new_tokens32000"}]</t>
+        </is>
+      </c>
+      <c r="K246" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0243</t>
+        </is>
+      </c>
+      <c r="B247" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="C247" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D247" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E247" s="10" t="inlineStr">
+        <is>
+          <t>77.2%</t>
+        </is>
+      </c>
+      <c r="F247" s="10" t="inlineStr"/>
+      <c r="G247" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H247" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml Performance / Cybersecurity / Footnotes</t>
+        </is>
+      </c>
+      <c r="I247" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym 77.2</t>
+        </is>
+      </c>
+      <c r="J247" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 77.2, "unit": "percent", "configuration": "GLM-5.3官方博客；独立模型列；1507题，single-run pass@1；GLM-5.3配置Claude Code2.1.207，max，无web，max_new_tokens128000；GLM-5.3主列不限任务超时；未单独披露GLM-5.2的完整配置，不将5.3设置自动归给5.2。"}]</t>
+        </is>
+      </c>
+      <c r="K247" s="10" t="inlineStr">
+        <is>
+          <t>后续同厂报告补测</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0244</t>
+        </is>
+      </c>
+      <c r="B248" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="C248" s="10" t="inlineStr">
+        <is>
+          <t>ExploitGym</t>
+        </is>
+      </c>
+      <c r="D248" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E248" s="10" t="inlineStr">
+        <is>
+          <t>2h:29题；6h:39题</t>
+        </is>
+      </c>
+      <c r="F248" s="10" t="inlineStr"/>
+      <c r="G248" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H248" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml Performance / Cybersecurity / Footnotes</t>
+        </is>
+      </c>
+      <c r="I248" s="10" t="inlineStr">
+        <is>
+          <t>ExploitGym 2h / 6h: 29 / 39; 869 tasks.</t>
+        </is>
+      </c>
+      <c r="J248" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "完成任务数", "value": 29, "unit": "count", "configuration": "GLM-5.3官方博客；独立模型列；869题；该项按模型吞吐归一化的时间预算；值为完成题数，不是百分比；2h预算"}, {"label": "完成任务数", "value": 39, "unit": "count", "configuration": "GLM-5.3官方博客；独立模型列；869题；该项按模型吞吐归一化的时间预算；值为完成题数，不是百分比；6h预算"}]</t>
+        </is>
+      </c>
+      <c r="K248" s="10" t="inlineStr">
+        <is>
+          <t>后续同厂报告补测</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0245</t>
+        </is>
+      </c>
+      <c r="B249" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="C249" s="10" t="inlineStr">
+        <is>
+          <t>ExploitBench</t>
+        </is>
+      </c>
+      <c r="D249" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E249" s="10" t="inlineStr">
+        <is>
+          <t>24.4%</t>
+        </is>
+      </c>
+      <c r="F249" s="10" t="inlineStr"/>
+      <c r="G249" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H249" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml Performance / Cybersecurity / Footnotes</t>
+        </is>
+      </c>
+      <c r="I249" s="10" t="inlineStr">
+        <is>
+          <t>ExploitBench 24.4%; average coverage score over all 41 tasks across 3 revisions; maximum 300 interaction rounds.</t>
+        </is>
+      </c>
+      <c r="J249" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "Cap%", "value": 24.4, "unit": "percent", "configuration": "GLM-5.3官方博客；独立模型列；能力覆盖分数；300轮；不可解释为完整代码执行成功率；41题，3 revisions取能力并集再平均；GLM-5.2完整设置未单独披露。"}]</t>
+        </is>
+      </c>
+      <c r="K249" s="10" t="inlineStr">
+        <is>
+          <t>后续同厂报告补测</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0246</t>
+        </is>
+      </c>
+      <c r="B250" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5.3</t>
+        </is>
+      </c>
+      <c r="C250" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D250" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E250" s="10" t="inlineStr">
+        <is>
+          <t>84.5%</t>
+        </is>
+      </c>
+      <c r="F250" s="10" t="inlineStr"/>
+      <c r="G250" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H250" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml Performance / Cybersecurity / Footnotes</t>
+        </is>
+      </c>
+      <c r="I250" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym 84.5</t>
+        </is>
+      </c>
+      <c r="J250" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 84.5, "unit": "percent", "configuration": "GLM-5.3官方博客；独立模型列；1507题，single-run pass@1；GLM-5.3配置Claude Code2.1.207，max，无web，max_new_tokens128000；GLM-5.3主列不限任务超时；未单独披露GLM-5.2的完整配置，不将5.3设置自动归给5.2。"}]</t>
+        </is>
+      </c>
+      <c r="K250" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0247</t>
+        </is>
+      </c>
+      <c r="B251" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5.3</t>
+        </is>
+      </c>
+      <c r="C251" s="10" t="inlineStr">
+        <is>
+          <t>ExploitGym</t>
+        </is>
+      </c>
+      <c r="D251" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E251" s="10" t="inlineStr">
+        <is>
+          <t>2h:105题；6h:130题</t>
+        </is>
+      </c>
+      <c r="F251" s="10" t="inlineStr"/>
+      <c r="G251" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H251" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml Performance / Cybersecurity / Footnotes</t>
+        </is>
+      </c>
+      <c r="I251" s="10" t="inlineStr">
+        <is>
+          <t>ExploitGym 2h / 6h: 105 / 130; 869 tasks.</t>
+        </is>
+      </c>
+      <c r="J251" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "完成任务数", "value": 105, "unit": "count", "configuration": "GLM-5.3官方博客；独立模型列；869题；该项按模型吞吐归一化的时间预算；值为完成题数，不是百分比；2h预算"}, {"label": "完成任务数", "value": 130, "unit": "count", "configuration": "GLM-5.3官方博客；独立模型列；869题；该项按模型吞吐归一化的时间预算；值为完成题数，不是百分比；6h预算"}]</t>
+        </is>
+      </c>
+      <c r="K251" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0248</t>
+        </is>
+      </c>
+      <c r="B252" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5.3</t>
+        </is>
+      </c>
+      <c r="C252" s="10" t="inlineStr">
+        <is>
+          <t>ExploitBench</t>
+        </is>
+      </c>
+      <c r="D252" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E252" s="10" t="inlineStr">
+        <is>
+          <t>54.4%</t>
+        </is>
+      </c>
+      <c r="F252" s="10" t="inlineStr"/>
+      <c r="G252" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H252" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml Performance / Cybersecurity / Footnotes</t>
+        </is>
+      </c>
+      <c r="I252" s="10" t="inlineStr">
+        <is>
+          <t>ExploitBench 54.4%; average coverage score over all 41 tasks across 3 revisions; maximum 300 interaction rounds.</t>
+        </is>
+      </c>
+      <c r="J252" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "Cap%", "value": 54.4, "unit": "percent", "configuration": "GLM-5.3官方博客；独立模型列；能力覆盖分数；300轮；不可解释为完整代码执行成功率；41题，3 revisions取能力并集再平均；GLM-5.2完整设置未单独披露。"}]</t>
+        </is>
+      </c>
+      <c r="K252" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0249</t>
+        </is>
+      </c>
+      <c r="B253" s="10" t="inlineStr">
+        <is>
+          <t>Grok 4.20</t>
+        </is>
+      </c>
+      <c r="C253" s="10" t="inlineStr">
+        <is>
+          <t>Cybench</t>
+        </is>
+      </c>
+      <c r="D253" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E253" s="10" t="inlineStr">
+        <is>
+          <t>53%</t>
+        </is>
+      </c>
+      <c r="F253" s="10" t="inlineStr"/>
+      <c r="G253" s="10" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="H253" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-20.pdf p.5-6</t>
+        </is>
+      </c>
+      <c r="I253" s="10" t="inlineStr">
+        <is>
+          <t>Table 4: Grok 4.2 SA — Cybench success rate 0.53</t>
+        </is>
+      </c>
+      <c r="J253" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "成功率", "value": 53, "unit": "percent", "configuration": "Grok 4.2 SA；防护前；unguided end-to-end；明确单Agent配置"}]</t>
+        </is>
+      </c>
+      <c r="K253" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0250</t>
+        </is>
+      </c>
+      <c r="B254" s="10" t="inlineStr">
+        <is>
+          <t>Grok 4.20</t>
+        </is>
+      </c>
+      <c r="C254" s="10" t="inlineStr">
+        <is>
+          <t>WMDP Cyber</t>
+        </is>
+      </c>
+      <c r="D254" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E254" s="10" t="inlineStr">
+        <is>
+          <t>91%</t>
+        </is>
+      </c>
+      <c r="F254" s="10" t="inlineStr"/>
+      <c r="G254" s="10" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="H254" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-20.pdf p.5</t>
+        </is>
+      </c>
+      <c r="I254" s="10" t="inlineStr">
+        <is>
+          <t>Table 4: Grok 4.2 SA — WMDP Cyber accuracy 0.91</t>
+        </is>
+      </c>
+      <c r="J254" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "准确率", "value": 91, "unit": "percent", "configuration": "Grok 4.2 SA；网安知识选择题；不能当作攻击任务成功率"}]</t>
+        </is>
+      </c>
+      <c r="K254" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0251</t>
+        </is>
+      </c>
+      <c r="B255" s="10" t="inlineStr">
+        <is>
+          <t>Grok 4.20 Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C255" s="10" t="inlineStr">
+        <is>
+          <t>Cybench / WMDP Cyber</t>
+        </is>
+      </c>
+      <c r="D255" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E255" s="10" t="inlineStr"/>
+      <c r="F255" s="10" t="inlineStr"/>
+      <c r="G255" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H255" s="10" t="inlineStr"/>
+      <c r="I255" s="10" t="inlineStr">
+        <is>
+          <t>模型覆盖待核对</t>
+        </is>
+      </c>
+      <c r="J255" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K255" s="10" t="inlineStr">
+        <is>
+          <t>模型覆盖待核对</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0252</t>
+        </is>
+      </c>
+      <c r="B256" s="10" t="inlineStr">
+        <is>
+          <t>Grok 4.20</t>
+        </is>
+      </c>
+      <c r="C256" s="10" t="inlineStr">
+        <is>
+          <t>AgentHarm</t>
+        </is>
+      </c>
+      <c r="D256" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E256" s="10" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="F256" s="10" t="inlineStr"/>
+      <c r="G256" s="10" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="H256" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-20.pdf p.3</t>
+        </is>
+      </c>
+      <c r="I256" s="10" t="inlineStr">
+        <is>
+          <t>Table 1: Grok 4.2 SA — AgentHarm violation rate 0.30; MA not reported.</t>
+        </is>
+      </c>
+      <c r="J256" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "违规率", "value": 30, "unit": "percent", "configuration": "恶意Agent任务拒答；含网安但也包含其他类别；不列为纯网安能力基准"}]</t>
+        </is>
+      </c>
+      <c r="K256" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0253</t>
+        </is>
+      </c>
+      <c r="B257" s="10" t="inlineStr">
+        <is>
+          <t>Grok 4.20</t>
+        </is>
+      </c>
+      <c r="C257" s="10" t="inlineStr">
+        <is>
+          <t>AgentDojo</t>
+        </is>
+      </c>
+      <c r="D257" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E257" s="10" t="inlineStr">
+        <is>
+          <t>33%</t>
+        </is>
+      </c>
+      <c r="F257" s="10" t="inlineStr"/>
+      <c r="G257" s="10" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="H257" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-20.pdf p.3</t>
+        </is>
+      </c>
+      <c r="I257" s="10" t="inlineStr">
+        <is>
+          <t>Table 1: Grok 4.2 SA — AgentDojo attack success rate 0.33; MA not reported.</t>
+        </is>
+      </c>
+      <c r="J257" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "攻击成功率", "value": 33, "unit": "percent", "configuration": "Agent提示注入鲁棒性；不等同网安攻击能力"}]</t>
+        </is>
+      </c>
+      <c r="K257" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0254</t>
+        </is>
+      </c>
+      <c r="B258" s="10" t="inlineStr">
+        <is>
+          <t>Grok 4.7</t>
+        </is>
+      </c>
+      <c r="C258" s="10" t="inlineStr">
+        <is>
+          <t>HackerBench v0.3</t>
+        </is>
+      </c>
+      <c r="D258" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E258" s="10" t="inlineStr">
+        <is>
+          <t>风险双用途提示放行率3.3%</t>
+        </is>
+      </c>
+      <c r="F258" s="10" t="inlineStr"/>
+      <c r="G258" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H258" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-7.html Safety &amp; Cybersecurity</t>
+        </is>
+      </c>
+      <c r="I258" s="10" t="inlineStr">
+        <is>
+          <t>allowing only 3.3% of risky dual-use prompts through</t>
+        </is>
+      </c>
+      <c r="J258" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "风险双用途提示放行率", "value": 3.3, "unit": "percent", "configuration": "网安风险请求安全性／拒答；越低越好，不是任务成功率"}]</t>
+        </is>
+      </c>
+      <c r="K258" s="10" t="inlineStr">
+        <is>
+          <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0255</t>
+        </is>
+      </c>
+      <c r="B259" s="10" t="inlineStr">
+        <is>
+          <t>Hy3</t>
+        </is>
+      </c>
+      <c r="C259" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D259" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E259" s="10" t="inlineStr">
+        <is>
+          <t>51.8%</t>
+        </is>
+      </c>
+      <c r="F259" s="10" t="inlineStr"/>
+      <c r="G259" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H259" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy3-benchmark-cybergym.html Benchmark Appendix / CyberGym行；sources/vendors/Tencent/hy4-benchmark-appendix.jpg CyberGym行／Hy3与Hy4 preview独立列</t>
+        </is>
+      </c>
+      <c r="I259" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym row: Hy3 51.8; Hy4 preview 78.4.
+CyberGym row: Hy3 51.8; Hy4 preview 78.4.</t>
+        </is>
+      </c>
+      <c r="J259" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 51.8, "unit": "percent", "configuration": "腾讯Hy4 preview官方模型卡基准附表；各模型最高可用推理设置；报告提醒Hy3部分成绩因harness、judge及反作弊机制更新而与旧报告不同"}]</t>
+        </is>
+      </c>
+      <c r="K259" s="10" t="inlineStr">
+        <is>
+          <t>后续官方报告补测；已人工核对官方图片；原表漏列。证据图片：docs/Tencent/hy4-benchmark-appendix.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0256</t>
+        </is>
+      </c>
+      <c r="B260" s="10" t="inlineStr">
+        <is>
+          <t>Hy4 preview</t>
+        </is>
+      </c>
+      <c r="C260" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D260" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E260" s="10" t="inlineStr">
+        <is>
+          <t>78.4%</t>
+        </is>
+      </c>
+      <c r="F260" s="10" t="inlineStr"/>
+      <c r="G260" s="10" t="inlineStr">
+        <is>
+          <t>official_web</t>
+        </is>
+      </c>
+      <c r="H260" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy3-benchmark-cybergym.html Benchmark Appendix / CyberGym行；sources/vendors/Tencent/hy4-benchmark-appendix.jpg CyberGym行／Hy3与Hy4 preview独立列</t>
+        </is>
+      </c>
+      <c r="I260" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym row: Hy3 51.8; Hy4 preview 78.4.
+CyberGym row: Hy3 51.8; Hy4 preview 78.4.</t>
+        </is>
+      </c>
+      <c r="J260" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 78.4, "unit": "percent", "configuration": "腾讯Hy4 preview官方模型卡基准附表；各模型最高可用推理设置；报告提醒Hy3部分成绩因harness、judge及反作弊机制更新而与旧报告不同"}]</t>
+        </is>
+      </c>
+      <c r="K260" s="10" t="inlineStr">
+        <is>
+          <t>已人工核对官方图片；原表漏列。证据图片：docs/Tencent/hy4-benchmark-appendix.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0257</t>
+        </is>
+      </c>
+      <c r="B261" s="10" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4.1-Flash-1017</t>
+        </is>
+      </c>
+      <c r="C261" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D261" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E261" s="10" t="inlineStr"/>
+      <c r="F261" s="10" t="inlineStr"/>
+      <c r="G261" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H261" s="10" t="inlineStr"/>
+      <c r="I261" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J261" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K261" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0258</t>
+        </is>
+      </c>
+      <c r="B262" s="10" t="inlineStr">
+        <is>
+          <t>GLM-4.7-Flash</t>
+        </is>
+      </c>
+      <c r="C262" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D262" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E262" s="10" t="inlineStr"/>
+      <c r="F262" s="10" t="inlineStr"/>
+      <c r="G262" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H262" s="10" t="inlineStr"/>
+      <c r="I262" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J262" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K262" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0259</t>
+        </is>
+      </c>
+      <c r="B263" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5-Turbo</t>
+        </is>
+      </c>
+      <c r="C263" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D263" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E263" s="10" t="inlineStr"/>
+      <c r="F263" s="10" t="inlineStr"/>
+      <c r="G263" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H263" s="10" t="inlineStr"/>
+      <c r="I263" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J263" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K263" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0260</t>
+        </is>
+      </c>
+      <c r="B264" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5V-Turbo</t>
+        </is>
+      </c>
+      <c r="C264" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D264" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E264" s="10" t="inlineStr"/>
+      <c r="F264" s="10" t="inlineStr"/>
+      <c r="G264" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H264" s="10" t="inlineStr"/>
+      <c r="I264" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J264" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K264" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0261</t>
+        </is>
+      </c>
+      <c r="B265" s="10" t="inlineStr">
+        <is>
+          <t>GLM-5.3-Flash</t>
+        </is>
+      </c>
+      <c r="C265" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D265" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E265" s="10" t="inlineStr"/>
+      <c r="F265" s="10" t="inlineStr"/>
+      <c r="G265" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H265" s="10" t="inlineStr"/>
+      <c r="I265" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J265" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K265" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0262</t>
+        </is>
+      </c>
+      <c r="B266" s="10" t="inlineStr">
+        <is>
+          <t>Hy3 preview</t>
+        </is>
+      </c>
+      <c r="C266" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D266" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E266" s="10" t="inlineStr"/>
+      <c r="F266" s="10" t="inlineStr"/>
+      <c r="G266" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H266" s="10" t="inlineStr"/>
+      <c r="I266" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J266" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K266" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0263</t>
+        </is>
+      </c>
+      <c r="B267" s="10" t="inlineStr">
+        <is>
+          <t>Grok Build 0.1</t>
+        </is>
+      </c>
+      <c r="C267" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D267" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E267" s="10" t="inlineStr"/>
+      <c r="F267" s="10" t="inlineStr"/>
+      <c r="G267" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H267" s="10" t="inlineStr"/>
+      <c r="I267" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J267" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K267" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0264</t>
+        </is>
+      </c>
+      <c r="B268" s="10" t="inlineStr">
+        <is>
+          <t>Grok 4.5</t>
+        </is>
+      </c>
+      <c r="C268" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D268" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E268" s="10" t="inlineStr"/>
+      <c r="F268" s="10" t="inlineStr"/>
+      <c r="G268" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H268" s="10" t="inlineStr"/>
+      <c r="I268" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J268" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K268" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0265</t>
+        </is>
+      </c>
+      <c r="B269" s="10" t="inlineStr">
+        <is>
+          <t>Grok 4.6</t>
+        </is>
+      </c>
+      <c r="C269" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D269" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E269" s="10" t="inlineStr"/>
+      <c r="F269" s="10" t="inlineStr"/>
+      <c r="G269" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H269" s="10" t="inlineStr"/>
+      <c r="I269" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J269" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K269" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0266</t>
+        </is>
+      </c>
+      <c r="B270" s="10" t="inlineStr">
+        <is>
+          <t>Grok 4.7 Fast</t>
+        </is>
+      </c>
+      <c r="C270" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D270" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E270" s="10" t="inlineStr"/>
+      <c r="F270" s="10" t="inlineStr"/>
+      <c r="G270" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H270" s="10" t="inlineStr"/>
+      <c r="I270" s="10" t="inlineStr">
+        <is>
+          <t>同模型服务档位</t>
+        </is>
+      </c>
+      <c r="J270" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K270" s="10" t="inlineStr">
+        <is>
+          <t>同模型服务档位</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0267</t>
+        </is>
+      </c>
+      <c r="B271" s="10" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Flash Preview</t>
+        </is>
+      </c>
+      <c r="C271" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D271" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E271" s="10" t="inlineStr"/>
+      <c r="F271" s="10" t="inlineStr"/>
+      <c r="G271" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H271" s="10" t="inlineStr"/>
+      <c r="I271" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J271" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K271" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0268</t>
+        </is>
+      </c>
+      <c r="B272" s="10" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Pro Preview</t>
+        </is>
+      </c>
+      <c r="C272" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D272" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E272" s="10" t="inlineStr"/>
+      <c r="F272" s="10" t="inlineStr"/>
+      <c r="G272" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H272" s="10" t="inlineStr"/>
+      <c r="I272" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J272" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K272" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:K237"/>
+  <autoFilter ref="A4:K272"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>模型ID</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>厂商</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>模型／版本</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>模型日期</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>日期精度</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>日期依据</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>日期说明</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>官方模型资料</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>本地归档</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>说明与限制</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>deepseek-v4-flash</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Flash</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-24（预览）；2026-07-31（正式版API公测）</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>PDF为V4系列共享卡，4月模型信息；7月正式版成绩以更新日志为准。 此条目按正式版日期绘图；4月预览版另列，不继承正式版成绩。</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/news/news260731/</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash.pdf</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>PDF为V4系列共享卡，4月模型信息；7月正式版成绩以更新日志为准。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>deepseek-v4-pro</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Pro</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-24（预览）；2026-08-13（正式版）</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>PDF为V4系列共享卡；正式版成绩以8月发布记录为准。 此条目按正式版日期绘图；4月预览版另列，不继承正式版成绩。</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/news/news260813/</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash.pdf</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="inlineStr">
+        <is>
+          <t>PDF为V4系列共享卡；正式版成绩以8月发布记录为准。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>deepseek-v4-flash-vision-exp</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Flash-Vision-Exp</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>已检查发布页基准图片：CyberGym 75.3，不继承Flash-0731的76.7。</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/news/news260821/</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-vision-exp.html</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>已检查发布页基准图片：CyberGym 75.3，不继承Flash-0731的76.7。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>deepseek-v4-1-flash</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4.1-Flash</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-10（发布）；2026-09-17（论文首发）</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>产品发布日期与后续技术报告日期分开。</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/DeepSeek-V4.1-Flash/resolve/main/DeepSeek_V41_Tech_Report.pdf</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-1-flash.pdf</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>产品发布日期与后续技术报告日期分开。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>deepseek-v4-1-flash-1017</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4.1-Flash-1017</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>已检查更新页图片及1017模型卡，未见该快照具名网安成绩；不继承9月版本。</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/news/news261017/</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-1-flash-1017.html</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>；9月V4.1技术报告不作为1017专属Model Card。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>glm-4-7-flash</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Zhipu</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>GLM-4.7-Flash</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>2026-01（发布月份）；2026-01-19（官方仓库创建时间，UTC）</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>仓库创建于2026-01-19T06:28:10Z；创建时间本身不能证明当时公开，不将它强行作为产品精确首发日。</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/zai-org/GLM-4.7-Flash</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-4-7-flash.html</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>仓库创建于2026-01-19T06:28:10Z；创建时间本身不能证明当时公开，不将它强行作为产品精确首发日。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>glm-5</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Zhipu</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>GLM-5</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>2026-02-12（官方发布页）；2026-02-17（论文首发）</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>模型发布日与论文提交日分开。</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2602.15763</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5.pdf</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>模型发布日与论文提交日分开。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>glm-5-turbo</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Zhipu</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>GLM-5-Turbo</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>2026-03（官方时间线）；原文03-15精确日待核</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>官方资料确认3月及模型用途；本次可访问的官方发布日志未保留03-15条目，不把原文精确日标为已确认。</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>https://docs.z.ai/guides/llm/glm-5-turbo</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-turbo.html</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>官方资料确认3月及模型用途；本次可访问的官方发布日志未保留03-15条目，不把原文精确日标为已确认。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>glm-5v-turbo</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Zhipu</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>GLM-5V-Turbo</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>2026-04（发布）；2026-04-02（官方仓库发布记录）；2026-04-29（论文首发）</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>原文04-01未由当前厂商一手来源确认；仓库明确记04-02，不把报告4月29日当首发日。</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2604.26752</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5v-turbo.pdf</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>原文04-01未由当前厂商一手来源确认；仓库明确记04-02，不把报告4月29日当首发日。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>glm-5-1</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Zhipu</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>GLM-5.1</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr"/>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>https://z.ai/blog/glm-5.1</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-1.mhtml</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>glm-5-2</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Zhipu</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>GLM-5.2</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr"/>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>https://z.ai/blog/glm-5.2</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-2.mhtml</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>glm-5-3</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Zhipu</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>GLM-5.3</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-14（宣布／Coding Plan）；2026-08-18（平台发布记录）</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>宣布、平台记录和开放权重是不同事件；博客说明权重计划在发布两周后开放，不推断精确开放日。</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>https://z.ai/blog/glm-5.3</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>宣布、平台记录和开放权重是不同事件；博客说明权重计划在发布两周后开放，不推断精确开放日。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>glm-5-3-flash</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Zhipu</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>GLM-5.3-Flash</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr"/>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>https://z.ai/blog/glm-5.3-flash</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3-flash.mhtml</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>hy3-preview</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Hy3 preview</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr"/>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>https://hunyuan.tencent.com/research/hy3-preview</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy3-preview.mhtml</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>hy3</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Hy3</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-06（正式发布）</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>已核正式发布日；原文“8月扩大国际访问”的精确事件日期未由本次主资料确认。</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>https://hunyuan.tencent.com/research/hy3</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy3.mhtml</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>已核对腾讯官方Hy4 preview基准附表图片，确认CyberGym；Hy3为后续报告中的比较结果，不归属于Hy3 preview。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>hy4-preview</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Hy4 preview</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr"/>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>https://github.com/Tencent-Hunyuan/Hy4-preview</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy4-preview.html</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>已核对腾讯官方Hy4 preview基准附表图片，确认CyberGym；独立模型列披露CyberGym。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>grok-4-20</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Grok 4.20</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-10（API上线）；2026-04-07（System Card）</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>System Card中“Grok 4.2 SA”指4.20的单Agent评测配置。</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>https://data.x.ai/2026-04-07-grok-4-20-model-card.pdf</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-20.pdf</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>System Card中“Grok 4.2 SA”指4.20的单Agent评测配置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>grok-4-20-multi-agent</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Grok 4.20 Multi-Agent</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-10（API上线）</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>共享System Card覆盖两种部署模式，但双用途表格仅报告SA；不得将SA网安成绩继承为MA成绩。</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>https://data.x.ai/2026-04-07-grok-4-20-model-card.pdf</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-20.pdf</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="inlineStr">
+        <is>
+          <t>共享System Card覆盖两种部署模式，但双用途表格仅报告SA；不得将SA网安成绩继承为MA成绩。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>grok-build-0-1</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Grok Build 0.1</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-19（API早期访问记录）；2026-05-29（API公测公告）</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr"/>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>https://x.ai/news/grok-build-0-1</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-build-0-1.html</t>
+        </is>
+      </c>
+      <c r="J20" s="12" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>grok-4-5</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Grok 4.5</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08（API上线）；2026-07-16（发布公告）</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr"/>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>https://x.ai/news/grok-4-5</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-5.html</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>grok-4-6</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Grok 4.6</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr"/>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>https://x.ai/news/grok-4-6</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-6.html</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>grok-4-7</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Grok 4.7</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>HackerBench v0.3的3.3%是风险提示放行率，不是网安任务成功率。</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>https://x.ai/news/grok-4-7</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-7.html</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="inlineStr">
+        <is>
+          <t>HackerBench v0.3的3.3%是风险提示放行率，不是网安任务成功率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>grok-4-7-fast</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Grok 4.7 Fast</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-21（服务档位）</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>官方发行说明明确Fast为同一模型，仅在Cursor和Grok Build提供；不作为独立模型重复计分。</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>https://x.ai/news/grok-4-7</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-7.html</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>官方发行说明明确Fast为同一模型，仅在Cursor和Grok Build提供；不作为独立模型重复计分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>deepseek-v4-flash-preview</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Flash Preview</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-24（预览）；2026-07-31（正式版API公测）</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>4月24日预览版；7月／8月正式版另列。共享V4模型卡未提供可归属的具名网安成绩。</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>https://fe-static.deepseek.com/chat/transparency/deepseek-V4-model-card-EN.pdf</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash.pdf</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>不得将正式版或其他型号的网安成绩继承为预览版成绩。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>deepseek-v4-pro-preview</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>DeepSeek-V4-Pro Preview</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-24（预览）；2026-08-13（正式版）</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>4月24日预览版；7月／8月正式版另列。共享V4模型卡未提供可归属的具名网安成绩。</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>https://fe-static.deepseek.com/chat/transparency/deepseek-V4-model-card-EN.pdf</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash.pdf</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>不得将正式版或其他型号的网安成绩继承为预览版成绩。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J26"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>文件</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>文件页数（非PDF为0）</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>SHA-256</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>官方来源</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>抓取时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-1-flash-1017.html</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>8125b7812df5c3bf3caf1dbddd2048381232970ea71dffd2df8b97bffc5f8c59</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/news/news261017/</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:27.289427+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-1-flash-release-2.html</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>2f884496b62a95aaf6a819374e5fed88d4be0f40c40cbab5dd7a3a866d5eb505</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/news/news260910/</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:27.288007+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-1-flash-release-3.html</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>20a85d60266362ba0213c8c523aad4229d8ecb75af2a55114bb7af3b4b7909c7</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2609.19969</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:35:12.758732+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-1-flash.pdf</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>ba68e2e40408125ae6d2f63a9a241b61c73910691c74ec1a2a7023c851eac08d</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/deepseek-ai/DeepSeek-V4.1-Flash/resolve/main/DeepSeek_V41_Tech_Report.pdf</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:34.240655+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-release-1.html</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>44aa1245d5d65d5fc54c8f47a9a3d3235e1ab064a8fc64d6a6e57f570ec8c99c</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/updates/</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:27.291022+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-release-2.html</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>5b940bd5a3f03d4e261e3e525278774f91d3b60f2fb3d6142303aae1133a7f1f</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/news/news260731/</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:27.287134+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash-vision-exp.html</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>9a9ec802743e123f83cbe5138790e2150024ce16ab80122ce1cc9d136405645a</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/news/news260821/</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:27.286896+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-flash.pdf</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>c225d71e3d3d21f263f6f4c2fda2f05757c61eb575a9d263cb9fee291576d5b0</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>https://fe-static.deepseek.com/chat/transparency/deepseek-V4-model-card-EN.pdf</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:32.677369+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/deepseek-v4-pro-release-2.html</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>136427cad4a383674473c7b32261ef6302464982718bcb4dccad6f56e0d7b76b</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/news/news260813/</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:27.286722+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/v4.1_261017_benchmark_table_en.png</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>官方基准表图片</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>52c22094008778b467230086bedb4faa4b846e70499307ee5da0c75fc3a15a01</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/img/v4.1_261017_benchmark_table_en.png</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/DeepSeek/v4_260821_benchmark_en.png</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>官方基准表图片</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>4b3cca9a4075fb05ad51cdc819e106d9baea19ac5f1ab38aa38a370c02bf26f3</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/img/v4_260821_benchmark_en.png</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy3-benchmark-cybergym.html</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>571ef5e97b9c766092a79a2d1dc370a3ce0855d29a18c958241efbf826b3801e</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/tencent/Hy4-preview</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T11:08:40.778487+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy3-preview.mhtml</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>c96cf9692bab99dd9b48512949840c9cfc0868e873b0195573a244c56524ebae</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>https://hunyuan.tencent.com/research/hy3-preview</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:34.783834+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy3.mhtml</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>df40271110ee6673a422cf8d3bcb10ebc2b353555f954156b33db31933cbd4b3</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>https://hunyuan.tencent.com/research/hy3</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:34.493614+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy4-benchmark-appendix.jpg</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>官方基准附表图片</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>02c751bf51c52c52cc02094561d7144bbfe3e27084d48d8a405d580da3554e21</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/tencent/Hy4-preview/resolve/main/assets/benchmark-appendix.jpg</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy4-preview-release-1.mhtml</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>e19b85f2f4349c0e39f6267b573479c22c268c400100e745fa49df72dada37f5</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>https://hunyuan.tencent.com/model/hy-model</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:34.276143+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Tencent/hy4-preview.html</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>f36851e5b4d27e8eff20f50480ec2d53a904bd8450f56ca6553f666a3483fbaa</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>https://github.com/Tencent-Hunyuan/Hy4-preview</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:27:51.739828+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-4-7-flash-release-1.html</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>831d4be1040cd91070eeec4fda43f82ae14412d270097f585458454400f9b1b4</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/api/models/zai-org/GLM-4.7-Flash</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:27:51.738340+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-4-7-flash.html</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>bcb2937e30f5fc2b6b45fb7bc585f7e9cdc64c5088627b6786cb5059d90c4298</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/zai-org/GLM-4.7-Flash</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:27:10.742095+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-1.mhtml</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>9eebe09595096b397431e64c60b20578a087e52442a7f2cc352d017a8c9ee957</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>https://z.ai/blog/glm-5.1</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:45.092784+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-2.mhtml</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>9d1569cd74e7b04e16fe00d19556159594f691b024eeb658d1c33c6298cb7951</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>https://z.ai/blog/glm-5.2</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:45.162698+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3-flash.mhtml</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>69cc57cac92ae7c0dd043f911dec37ad8fb6c862fde0b45b99ef634de456ade1</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>https://z.ai/blog/glm-5.3-flash</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:45.181770+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>b3e0c6d51c6c4948207694bfc4bb216ff5fd2075e614af730aa991e4329f4882</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>https://z.ai/blog/glm-5.3</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:45.166224+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-release-1.mhtml</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>d0c9e42034b0dc2f6edfcbeb96fa41fad376a48ca2ff4fd8543a88e6b9e828cd</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>https://z.ai/blog/glm-5</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:44.685558+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-turbo-release-1.html</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>f670bffaa05b62460258e9c49f7192dab32a772dd87f59db9e6a5133b13e3bda</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>https://autoclaw.z.ai/models/</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:29:59.255240+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-turbo.html</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>f189a2f083ddbfe76163462ab48ee340a898cacf9ef44623afe2082c29500fde</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>https://docs.z.ai/guides/llm/glm-5-turbo</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:27:10.740270+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5.pdf</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>e20742ff36e08dc361de6973f7f72ad38e107edf8fd92d2a777a8428fc9b8f0e</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2602.15763</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:27:10.745237+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5v-turbo-release-1.html</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>eb45372dab7e901d45f56892912e857914f4ef033fb8d17fcf80dafa275e004f</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>https://github.com/zai-org/GLM-V</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:27:10.743064+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5v-turbo.pdf</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>c6a28b9f33039e0324cb04cedad322dfbf55f23f9b7b0554480b788b4c22b834</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2604.26752</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:27:10.744104+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/zai-release-notes.html</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>a97ee4c68b2057d2878f496f0717ca07393d6860fdc40f05f92cb7d592cffdc5</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>https://docs.z.ai/release-notes/new-released</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:28:36.340991+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-20.pdf</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>ea72c27a6b04949d07c828b1dc5971688a79a780e5727eeca1985434d3262760</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>https://data.x.ai/2026-04-07-grok-4-20-model-card.pdf</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:28.333446+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-5.html</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>f4da93a6d5eb4a2e7a57c79e566478e67fa4cc136e7b2f48dce1681f0b9acff2</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>https://x.ai/news/grok-4-5</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:43.864933+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-6.html</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>24d0b48b966e0177d15c51ad106efad1da5ae72ee6ace7f5d26cb8eb486d7960</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>https://x.ai/news/grok-4-6</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:43.873709+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-4-7.html</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>ad8620db889ba6478a156599375a550d35218d075e5b6f02a9917ac598ce989f</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>https://x.ai/news/grok-4-7</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:44.385178+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/grok-build-0-1.html</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>1812731dcff815bfbe871aa7339c1da0eb7cebb88ec10bb3f59ef8d6101fff07</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>https://x.ai/news/grok-build-0-1</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:44.465111+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/xAI/xai-release-notes.html</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>345795792cc0152dd3cfc5fbb780e141a040fb840ffd70a6a50ced269cf16bd3</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>https://docs.x.ai/developers/release-notes</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:25:32.382055+00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Kimi models, sourced cyber evaluations, reports and logo
</commit_message>
<xml_diff>
--- a/web/public/downloads/audit-2026-10-18.xlsx
+++ b/web/public/downloads/audit-2026-10-18.xlsx
@@ -42,9 +42,9 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'修订记录'!$1:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'访问日志'!$A$4:$H$108</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'访问日志'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'成绩补录审计'!$A$4:$K$272</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'新增厂商模型'!$A$1:$J$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'新增厂商证据文件'!$A$1:$F$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'成绩补录审计'!$A$4:$M$286</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'新增厂商模型'!$A$1:$J$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'新增厂商证据文件'!$A$1:$F$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -994,7 +994,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>新增腾讯、智谱GLM、DeepSeek、xAI共25个模型／版本、35条记录；网页和图片以章节／表格定位，不伪造PDF页码。所有记录见成绩补录审计表，新增模型和证据文件另列。</t>
+          <t>新增腾讯、智谱GLM、DeepSeek、xAI、Kimi共31个模型／版本、49条记录；网页和图片以章节／表格定位，不伪造PDF页码。所有记录见成绩补录审计表，新增模型和证据文件另列。Kimi区分厂商自测、其他厂商比较和独立机构评测。</t>
         </is>
       </c>
     </row>
@@ -5270,7 +5270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K272"/>
+  <dimension ref="A1:M286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5284,6 +5284,8 @@
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5302,11 +5304,13 @@
       <c r="I1" s="10" t="n"/>
       <c r="J1" s="10" t="n"/>
       <c r="K1" s="10" t="n"/>
+      <c r="L1" s="10" t="n"/>
+      <c r="M1" s="10" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>复核218条已确认记录；原成绩43条，现已核实数值178条，新增数值135条。</t>
+          <t>复核229条已确认记录；原成绩43条，现已核实数值189条，新增数值146条。</t>
         </is>
       </c>
       <c r="B2" s="10" t="n"/>
@@ -5319,6 +5323,8 @@
       <c r="I2" s="10" t="n"/>
       <c r="J2" s="10" t="n"/>
       <c r="K2" s="10" t="n"/>
+      <c r="L2" s="10" t="n"/>
+      <c r="M2" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="n"/>
@@ -5332,6 +5338,8 @@
       <c r="I3" s="10" t="n"/>
       <c r="J3" s="10" t="n"/>
       <c r="K3" s="10" t="n"/>
+      <c r="L3" s="10" t="n"/>
+      <c r="M3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -5389,6 +5397,16 @@
           <t>备注</t>
         </is>
       </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>评测方</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>评测来源类型</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -5442,6 +5460,8 @@
           <t>图5当前模型柱标88%；不得用后续报告更精细的88.2%覆盖本报告原值。</t>
         </is>
       </c>
+      <c r="L5" s="10" t="inlineStr"/>
+      <c r="M5" s="10" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -5499,6 +5519,8 @@
           <t>核验原有90%正确；34/40题，zero-day、无源码，3 rollouts。</t>
         </is>
       </c>
+      <c r="L6" s="10" t="inlineStr"/>
+      <c r="M6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -5556,6 +5578,8 @@
           <t>15个场景，每场景16次尝试中至少成功一次计通过。</t>
         </is>
       </c>
+      <c r="L7" s="10" t="inlineStr"/>
+      <c r="M7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -5601,6 +5625,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L8" s="10" t="inlineStr"/>
+      <c r="M8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -5646,6 +5672,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L9" s="10" t="inlineStr"/>
+      <c r="M9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -5695,6 +5723,8 @@
         </is>
       </c>
       <c r="K10" s="10" t="inlineStr"/>
+      <c r="L10" s="10" t="inlineStr"/>
+      <c r="M10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -5744,6 +5774,8 @@
         </is>
       </c>
       <c r="K11" s="10" t="inlineStr"/>
+      <c r="L11" s="10" t="inlineStr"/>
+      <c r="M11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -5793,6 +5825,8 @@
         </is>
       </c>
       <c r="K12" s="10" t="inlineStr"/>
+      <c r="L12" s="10" t="inlineStr"/>
+      <c r="M12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -5846,6 +5880,8 @@
           <t>近最终代表性checkpoint，high reasoning，每题最多1000 turns，100K tokens compaction。</t>
         </is>
       </c>
+      <c r="L13" s="10" t="inlineStr"/>
+      <c r="M13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -5899,6 +5935,8 @@
         </is>
       </c>
       <c r="K14" s="10" t="inlineStr"/>
+      <c r="L14" s="10" t="inlineStr"/>
+      <c r="M14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -5944,6 +5982,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L15" s="10" t="inlineStr"/>
+      <c r="M15" s="10" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -5989,6 +6029,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L16" s="10" t="inlineStr"/>
+      <c r="M16" s="10" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -6034,6 +6076,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L17" s="10" t="inlineStr"/>
+      <c r="M17" s="10" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -6087,6 +6131,8 @@
         </is>
       </c>
       <c r="K18" s="10" t="inlineStr"/>
+      <c r="L18" s="10" t="inlineStr"/>
+      <c r="M18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -6140,6 +6186,8 @@
         </is>
       </c>
       <c r="K19" s="10" t="inlineStr"/>
+      <c r="L19" s="10" t="inlineStr"/>
+      <c r="M19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -6185,6 +6233,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L20" s="10" t="inlineStr"/>
+      <c r="M20" s="10" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -6230,6 +6280,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L21" s="10" t="inlineStr"/>
+      <c r="M21" s="10" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
@@ -6279,6 +6331,8 @@
         </is>
       </c>
       <c r="K22" s="10" t="inlineStr"/>
+      <c r="L22" s="10" t="inlineStr"/>
+      <c r="M22" s="10" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
@@ -6328,6 +6382,8 @@
         </is>
       </c>
       <c r="K23" s="10" t="inlineStr"/>
+      <c r="L23" s="10" t="inlineStr"/>
+      <c r="M23" s="10" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -6377,6 +6433,8 @@
         </is>
       </c>
       <c r="K24" s="10" t="inlineStr"/>
+      <c r="L24" s="10" t="inlineStr"/>
+      <c r="M24" s="10" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
@@ -6426,6 +6484,8 @@
           <t>有可信memory-safety线索及部分受控利用primitive；仅定性披露，不能将未达Critical当作0分。</t>
         </is>
       </c>
+      <c r="L25" s="10" t="inlineStr"/>
+      <c r="M25" s="10" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -6479,6 +6539,8 @@
         </is>
       </c>
       <c r="K26" s="10" t="inlineStr"/>
+      <c r="L26" s="10" t="inlineStr"/>
+      <c r="M26" s="10" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
@@ -6532,6 +6594,8 @@
           <t>本报告写all atomic challenges，不从其他版本补入任务数。后续5.6报告给GPT-5.5网络攻击模拟100%，与本报告98%不同，保留原值。</t>
         </is>
       </c>
+      <c r="L27" s="10" t="inlineStr"/>
+      <c r="M27" s="10" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
@@ -6581,6 +6645,8 @@
           <t>CAISI同时获得代表性发布checkpoint及降低拒答checkpoint；专家探测混用两者，只给相对结论。</t>
         </is>
       </c>
+      <c r="L28" s="10" t="inlineStr"/>
+      <c r="M28" s="10" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
@@ -6634,6 +6700,8 @@
           <t>代表性发布及降低拒答checkpoint；最高记录3/10不是统一重复实验均值，保留单独描述。另一个工业控制range未解。</t>
         </is>
       </c>
+      <c r="L29" s="10" t="inlineStr"/>
+      <c r="M29" s="10" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
@@ -6687,6 +6755,8 @@
         </is>
       </c>
       <c r="K30" s="10" t="inlineStr"/>
+      <c r="L30" s="10" t="inlineStr"/>
+      <c r="M30" s="10" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -6732,6 +6802,8 @@
           <t>明确未运行</t>
         </is>
       </c>
+      <c r="L31" s="10" t="inlineStr"/>
+      <c r="M31" s="10" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
@@ -6781,6 +6853,8 @@
         </is>
       </c>
       <c r="K32" s="10" t="inlineStr"/>
+      <c r="L32" s="10" t="inlineStr"/>
+      <c r="M32" s="10" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
@@ -6826,6 +6900,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L33" s="10" t="inlineStr"/>
+      <c r="M33" s="10" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
@@ -6871,6 +6947,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L34" s="10" t="inlineStr"/>
+      <c r="M34" s="10" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -6920,6 +6998,8 @@
         </is>
       </c>
       <c r="K35" s="10" t="inlineStr"/>
+      <c r="L35" s="10" t="inlineStr"/>
+      <c r="M35" s="10" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -6969,6 +7049,8 @@
         </is>
       </c>
       <c r="K36" s="10" t="inlineStr"/>
+      <c r="L36" s="10" t="inlineStr"/>
+      <c r="M36" s="10" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
@@ -7022,6 +7104,8 @@
           <t>本表13个场景，剔除了Printer Queue和Simple Privilege Escalation；不可和GPT-5.5原报告15场景93.33%直接比较。</t>
         </is>
       </c>
+      <c r="L37" s="10" t="inlineStr"/>
+      <c r="M37" s="10" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -7075,6 +7159,8 @@
           <t>图30精确柱标；正文Sol四舍五入为96.7%。63题新版CTF，不能与旧Professional pass@12混比。该预览报告图中模型标签写GPT-5.6 Sol，记录保留原有preview报告快照身份。</t>
         </is>
       </c>
+      <c r="L38" s="10" t="inlineStr"/>
+      <c r="M38" s="10" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -7124,6 +7210,8 @@
           <t>已查看图32；34/40题、zero-day、无源码、3 rollouts。图只有曲线，不能用刻度估读精确分数。</t>
         </is>
       </c>
+      <c r="L39" s="10" t="inlineStr"/>
+      <c r="M39" s="10" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -7173,6 +7261,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L40" s="10" t="inlineStr"/>
+      <c r="M40" s="10" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -7222,6 +7312,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L41" s="10" t="inlineStr"/>
+      <c r="M41" s="10" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
@@ -7271,6 +7363,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L42" s="10" t="inlineStr"/>
+      <c r="M42" s="10" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
@@ -7320,6 +7414,8 @@
           <t>多日研究产生真实PoC与受控利用primitive；仅定性披露，不把未达Critical当成0%。</t>
         </is>
       </c>
+      <c r="L43" s="10" t="inlineStr"/>
+      <c r="M43" s="10" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
@@ -7373,6 +7469,8 @@
           <t>Irregular harness，分母受设备可用性影响，不同模型略异。百分比保留报告四舍五入原值。</t>
         </is>
       </c>
+      <c r="L44" s="10" t="inlineStr"/>
+      <c r="M44" s="10" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
@@ -7422,6 +7520,8 @@
         </is>
       </c>
       <c r="K45" s="10" t="inlineStr"/>
+      <c r="L45" s="10" t="inlineStr"/>
+      <c r="M45" s="10" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
@@ -7471,6 +7571,8 @@
         </is>
       </c>
       <c r="K46" s="10" t="inlineStr"/>
+      <c r="L46" s="10" t="inlineStr"/>
+      <c r="M46" s="10" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
@@ -7524,6 +7626,8 @@
           <t>图30精确柱标；正文Sol四舍五入为96.7%。63题新版CTF，不能与旧Professional pass@12混比。</t>
         </is>
       </c>
+      <c r="L47" s="10" t="inlineStr"/>
+      <c r="M47" s="10" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
@@ -7573,6 +7677,8 @@
           <t>已查看图32；34/40题、zero-day、无源码、3 rollouts。图只有曲线，不能用刻度估读精确分数。</t>
         </is>
       </c>
+      <c r="L48" s="10" t="inlineStr"/>
+      <c r="M48" s="10" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
@@ -7622,6 +7728,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L49" s="10" t="inlineStr"/>
+      <c r="M49" s="10" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
@@ -7671,6 +7779,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L50" s="10" t="inlineStr"/>
+      <c r="M50" s="10" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
@@ -7720,6 +7830,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L51" s="10" t="inlineStr"/>
+      <c r="M51" s="10" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
@@ -7769,6 +7881,8 @@
           <t>多日研究产生真实PoC与受控利用primitive；仅定性披露，不把未达Critical当成0%。</t>
         </is>
       </c>
+      <c r="L52" s="10" t="inlineStr"/>
+      <c r="M52" s="10" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
@@ -7822,6 +7936,8 @@
           <t>Irregular harness，分母受设备可用性影响，不同模型略异。百分比保留报告四舍五入原值。</t>
         </is>
       </c>
+      <c r="L53" s="10" t="inlineStr"/>
+      <c r="M53" s="10" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
@@ -7871,6 +7987,8 @@
         </is>
       </c>
       <c r="K54" s="10" t="inlineStr"/>
+      <c r="L54" s="10" t="inlineStr"/>
+      <c r="M54" s="10" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
@@ -7920,6 +8038,8 @@
         </is>
       </c>
       <c r="K55" s="10" t="inlineStr"/>
+      <c r="L55" s="10" t="inlineStr"/>
+      <c r="M55" s="10" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
@@ -7973,6 +8093,8 @@
           <t>图30精确柱标；正文Sol四舍五入为96.7%。63题新版CTF，不能与旧Professional pass@12混比。</t>
         </is>
       </c>
+      <c r="L56" s="10" t="inlineStr"/>
+      <c r="M56" s="10" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
@@ -8022,6 +8144,8 @@
           <t>已查看图32；34/40题、zero-day、无源码、3 rollouts。图只有曲线，不能用刻度估读精确分数。</t>
         </is>
       </c>
+      <c r="L57" s="10" t="inlineStr"/>
+      <c r="M57" s="10" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
@@ -8071,6 +8195,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L58" s="10" t="inlineStr"/>
+      <c r="M58" s="10" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
@@ -8120,6 +8246,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L59" s="10" t="inlineStr"/>
+      <c r="M59" s="10" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
@@ -8169,6 +8297,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L60" s="10" t="inlineStr"/>
+      <c r="M60" s="10" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
@@ -8214,6 +8344,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L61" s="10" t="inlineStr"/>
+      <c r="M61" s="10" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
@@ -8267,6 +8399,8 @@
           <t>图30精确柱标；正文Sol四舍五入为96.7%。63题新版CTF，不能与旧Professional pass@12混比。</t>
         </is>
       </c>
+      <c r="L62" s="10" t="inlineStr"/>
+      <c r="M62" s="10" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
@@ -8316,6 +8450,8 @@
           <t>已查看图32；34/40题、zero-day、无源码、3 rollouts。图只有曲线，不能用刻度估读精确分数。</t>
         </is>
       </c>
+      <c r="L63" s="10" t="inlineStr"/>
+      <c r="M63" s="10" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
@@ -8365,6 +8501,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L64" s="10" t="inlineStr"/>
+      <c r="M64" s="10" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
@@ -8414,6 +8552,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L65" s="10" t="inlineStr"/>
+      <c r="M65" s="10" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
@@ -8463,6 +8603,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L66" s="10" t="inlineStr"/>
+      <c r="M66" s="10" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
@@ -8508,6 +8650,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L67" s="10" t="inlineStr"/>
+      <c r="M67" s="10" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
@@ -8561,6 +8705,8 @@
           <t>保留进度指标，不将3/10当成Doing Life完成率。</t>
         </is>
       </c>
+      <c r="L68" s="10" t="inlineStr"/>
+      <c r="M68" s="10" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
@@ -8618,6 +8764,8 @@
           <t>更新评分：任一种子达ACE即16/16满分；最低测试reasoning已满分；可能历史漏洞污染。</t>
         </is>
       </c>
+      <c r="L69" s="10" t="inlineStr"/>
+      <c r="M69" s="10" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
@@ -8672,6 +8820,8 @@
           <t>附录图80及正文精确31.5%，对应近期漏洞内部移植集比较。主报告图47同时给增加API攻击面与缩减API攻击面两条曲线但未逐点标值；不可将31.5%用于新增API攻击面曲线。</t>
         </is>
       </c>
+      <c r="L70" s="10" t="inlineStr"/>
+      <c r="M70" s="10" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
@@ -8725,6 +8875,8 @@
           <t>增加root-cause审计grader，不能与5.6原公开grader直接混比。</t>
         </is>
       </c>
+      <c r="L71" s="10" t="inlineStr"/>
+      <c r="M71" s="10" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
@@ -8778,6 +8930,8 @@
           <t>updated v1 implementation，运行时禁装包、离线、token cap无wall-clock cap。</t>
         </is>
       </c>
+      <c r="L72" s="10" t="inlineStr"/>
+      <c r="M72" s="10" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
@@ -8835,6 +8989,8 @@
           <t>补齐原表只保留的pass@4之外的pass@1。262 binaries、19私有程序，六个目标全部满足才通过。</t>
         </is>
       </c>
+      <c r="L73" s="10" t="inlineStr"/>
+      <c r="M73" s="10" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
@@ -8888,6 +9044,8 @@
         </is>
       </c>
       <c r="K74" s="10" t="inlineStr"/>
+      <c r="L74" s="10" t="inlineStr"/>
+      <c r="M74" s="10" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
@@ -8941,6 +9099,8 @@
           <t>专家仅安全监督/验证；Codex Ultra，最多64 subagents。时间不是成功率；不将初始缺防护build当成稳定版成绩。</t>
         </is>
       </c>
+      <c r="L75" s="10" t="inlineStr"/>
+      <c r="M75" s="10" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
@@ -8994,6 +9154,8 @@
           <t>Irregular沙箱、无公开互联网。</t>
         </is>
       </c>
+      <c r="L76" s="10" t="inlineStr"/>
+      <c r="M76" s="10" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
@@ -9043,6 +9205,8 @@
         </is>
       </c>
       <c r="K77" s="10" t="inlineStr"/>
+      <c r="L77" s="10" t="inlineStr"/>
+      <c r="M77" s="10" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
@@ -9092,6 +9256,8 @@
         </is>
       </c>
       <c r="K78" s="10" t="inlineStr"/>
+      <c r="L78" s="10" t="inlineStr"/>
+      <c r="M78" s="10" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
@@ -9145,6 +9311,8 @@
           <t>September报告附录值，保留该版本与配置。</t>
         </is>
       </c>
+      <c r="L79" s="10" t="inlineStr"/>
+      <c r="M79" s="10" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
@@ -9198,6 +9366,8 @@
           <t>September报告附录值，保留该版本与配置。</t>
         </is>
       </c>
+      <c r="L80" s="10" t="inlineStr"/>
+      <c r="M80" s="10" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
@@ -9251,6 +9421,8 @@
           <t>September报告附录值，保留该版本与配置。</t>
         </is>
       </c>
+      <c r="L81" s="10" t="inlineStr"/>
+      <c r="M81" s="10" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
@@ -9304,6 +9476,8 @@
           <t>September报告附录值，保留该版本与配置。</t>
         </is>
       </c>
+      <c r="L82" s="10" t="inlineStr"/>
+      <c r="M82" s="10" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
@@ -9353,6 +9527,8 @@
         </is>
       </c>
       <c r="K83" s="10" t="inlineStr"/>
+      <c r="L83" s="10" t="inlineStr"/>
+      <c r="M83" s="10" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
@@ -9406,6 +9582,8 @@
           <t>September报告附录值，保留该版本与配置。</t>
         </is>
       </c>
+      <c r="L84" s="10" t="inlineStr"/>
+      <c r="M84" s="10" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
@@ -9459,6 +9637,8 @@
           <t>September报告附录值，保留该版本与配置。</t>
         </is>
       </c>
+      <c r="L85" s="10" t="inlineStr"/>
+      <c r="M85" s="10" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
@@ -9512,6 +9692,8 @@
           <t>September报告附录值，保留该版本与配置。</t>
         </is>
       </c>
+      <c r="L86" s="10" t="inlineStr"/>
+      <c r="M86" s="10" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
@@ -9565,6 +9747,8 @@
           <t>September报告附录值，保留该版本与配置。</t>
         </is>
       </c>
+      <c r="L87" s="10" t="inlineStr"/>
+      <c r="M87" s="10" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
@@ -9614,6 +9798,8 @@
         </is>
       </c>
       <c r="K88" s="10" t="inlineStr"/>
+      <c r="L88" s="10" t="inlineStr"/>
+      <c r="M88" s="10" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
@@ -9667,6 +9853,8 @@
         </is>
       </c>
       <c r="K89" s="10" t="inlineStr"/>
+      <c r="L89" s="10" t="inlineStr"/>
+      <c r="M89" s="10" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
@@ -9720,6 +9908,8 @@
         </is>
       </c>
       <c r="K90" s="10" t="inlineStr"/>
+      <c r="L90" s="10" t="inlineStr"/>
+      <c r="M90" s="10" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
@@ -9765,6 +9955,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L91" s="10" t="inlineStr"/>
+      <c r="M91" s="10" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
@@ -9810,6 +10002,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L92" s="10" t="inlineStr"/>
+      <c r="M92" s="10" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
@@ -9855,6 +10049,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L93" s="10" t="inlineStr"/>
+      <c r="M93" s="10" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
@@ -9908,6 +10104,8 @@
         </is>
       </c>
       <c r="K94" s="10" t="inlineStr"/>
+      <c r="L94" s="10" t="inlineStr"/>
+      <c r="M94" s="10" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
@@ -9961,6 +10159,8 @@
         </is>
       </c>
       <c r="K95" s="10" t="inlineStr"/>
+      <c r="L95" s="10" t="inlineStr"/>
+      <c r="M95" s="10" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
@@ -10006,6 +10206,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L96" s="10" t="inlineStr"/>
+      <c r="M96" s="10" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
@@ -10051,6 +10253,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L97" s="10" t="inlineStr"/>
+      <c r="M97" s="10" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
@@ -10096,6 +10300,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L98" s="10" t="inlineStr"/>
+      <c r="M98" s="10" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
@@ -10149,6 +10355,8 @@
         </is>
       </c>
       <c r="K99" s="10" t="inlineStr"/>
+      <c r="L99" s="10" t="inlineStr"/>
+      <c r="M99" s="10" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
@@ -10202,6 +10410,8 @@
         </is>
       </c>
       <c r="K100" s="10" t="inlineStr"/>
+      <c r="L100" s="10" t="inlineStr"/>
+      <c r="M100" s="10" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
@@ -10255,6 +10465,8 @@
         </is>
       </c>
       <c r="K101" s="10" t="inlineStr"/>
+      <c r="L101" s="10" t="inlineStr"/>
+      <c r="M101" s="10" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
@@ -10308,6 +10520,8 @@
         </is>
       </c>
       <c r="K102" s="10" t="inlineStr"/>
+      <c r="L102" s="10" t="inlineStr"/>
+      <c r="M102" s="10" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
@@ -10353,6 +10567,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L103" s="10" t="inlineStr"/>
+      <c r="M103" s="10" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
@@ -10410,6 +10626,8 @@
           <t>2026-06-22完整版本更新，单模型发布文章数值。</t>
         </is>
       </c>
+      <c r="L104" s="10" t="inlineStr"/>
+      <c r="M104" s="10" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
@@ -10467,6 +10685,8 @@
           <t>2026-06-22完整版本更新，单模型发布文章数值。</t>
         </is>
       </c>
+      <c r="L105" s="10" t="inlineStr"/>
+      <c r="M105" s="10" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
@@ -10524,6 +10744,8 @@
           <t>2026-06-22完整版本更新，单模型发布文章数值。</t>
         </is>
       </c>
+      <c r="L106" s="10" t="inlineStr"/>
+      <c r="M106" s="10" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
@@ -10573,6 +10795,8 @@
           <t>已查看网页转制PDF正文及页面图像：该项仅披露相对结论，未给精确分数；不得挪用6月另一配置ExploitGym 39.5%。最高公开reasoning；内部加固实现。</t>
         </is>
       </c>
+      <c r="L107" s="10" t="inlineStr"/>
+      <c r="M107" s="10" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
@@ -10626,6 +10850,8 @@
           <t>Daybreak Red；衡量模型回应高级网安请求的比例，不是任务成功率。</t>
         </is>
       </c>
+      <c r="L108" s="10" t="inlineStr"/>
+      <c r="M108" s="10" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
@@ -10675,6 +10901,8 @@
           <t>已查看网页转制PDF正文及页面图像：该项仅披露相对结论，未给精确分数；不得挪用6月另一配置ExploitGym 39.5%。最高公开reasoning；内部加固实现。</t>
         </is>
       </c>
+      <c r="L109" s="10" t="inlineStr"/>
+      <c r="M109" s="10" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
@@ -10724,6 +10952,8 @@
           <t>已查看网页转制PDF正文及页面图像：该项仅披露相对结论，未给精确分数；不得挪用6月另一配置ExploitGym 39.5%。最高公开reasoning；内部加固实现。</t>
         </is>
       </c>
+      <c r="L110" s="10" t="inlineStr"/>
+      <c r="M110" s="10" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
@@ -10777,6 +11007,8 @@
           <t>Daybreak Red；衡量模型回应高级网安请求的比例，不是任务成功率。</t>
         </is>
       </c>
+      <c r="L111" s="10" t="inlineStr"/>
+      <c r="M111" s="10" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
@@ -10826,6 +11058,8 @@
           <t>已查看网页转制PDF正文及页面图像：该项仅披露相对结论，未给精确分数；不得挪用6月另一配置ExploitGym 39.5%。最高公开reasoning；内部加固实现。</t>
         </is>
       </c>
+      <c r="L112" s="10" t="inlineStr"/>
+      <c r="M112" s="10" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
@@ -10875,6 +11109,8 @@
           <t>已查看网页转制PDF正文及页面图像：该项仅披露相对结论，未给精确分数；不得挪用6月另一配置ExploitGym 39.5%。最高公开reasoning；内部加固实现。</t>
         </is>
       </c>
+      <c r="L113" s="10" t="inlineStr"/>
+      <c r="M113" s="10" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
@@ -10924,6 +11160,8 @@
           <t>已查看网页转制PDF正文及页面图像：该项仅披露相对结论，未给精确分数；不得挪用6月另一配置ExploitGym 39.5%。最高公开reasoning；内部加固实现。</t>
         </is>
       </c>
+      <c r="L114" s="10" t="inlineStr"/>
+      <c r="M114" s="10" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
@@ -10973,6 +11211,8 @@
         </is>
       </c>
       <c r="K115" s="10" t="inlineStr"/>
+      <c r="L115" s="10" t="inlineStr"/>
+      <c r="M115" s="10" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
@@ -11026,6 +11266,8 @@
           <t>原卡称未运行40题中的3题，原表35/40配置不能直接套用；后续卡纠正判分后为1.00，不覆盖本条原始结果。</t>
         </is>
       </c>
+      <c r="L116" s="10" t="inlineStr"/>
+      <c r="M116" s="10" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
@@ -11079,6 +11321,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L117" s="10" t="inlineStr"/>
+      <c r="M117" s="10" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
@@ -11132,6 +11376,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L118" s="10" t="inlineStr"/>
+      <c r="M118" s="10" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
@@ -11185,6 +11431,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L119" s="10" t="inlineStr"/>
+      <c r="M119" s="10" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
@@ -11238,6 +11486,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L120" s="10" t="inlineStr"/>
+      <c r="M120" s="10" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
@@ -11291,6 +11541,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L121" s="10" t="inlineStr"/>
+      <c r="M121" s="10" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
@@ -11340,6 +11592,8 @@
         </is>
       </c>
       <c r="K122" s="10" t="inlineStr"/>
+      <c r="L122" s="10" t="inlineStr"/>
+      <c r="M122" s="10" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
@@ -11393,6 +11647,8 @@
           <t>原卡称未运行40题中的3题；后续纠正判分为0.96，不覆盖本条。</t>
         </is>
       </c>
+      <c r="L123" s="10" t="inlineStr"/>
+      <c r="M123" s="10" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
@@ -11446,6 +11702,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L124" s="10" t="inlineStr"/>
+      <c r="M124" s="10" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
@@ -11499,6 +11757,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L125" s="10" t="inlineStr"/>
+      <c r="M125" s="10" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
@@ -11552,6 +11812,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L126" s="10" t="inlineStr"/>
+      <c r="M126" s="10" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
@@ -11605,6 +11867,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L127" s="10" t="inlineStr"/>
+      <c r="M127" s="10" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
@@ -11658,6 +11922,8 @@
           <t>分母采用结果图与图注，和Details段所列题目数不同；不得当作单次成功率。</t>
         </is>
       </c>
+      <c r="L128" s="10" t="inlineStr"/>
+      <c r="M128" s="10" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
@@ -11707,6 +11973,8 @@
           <t>报告描述发现多个新漏洞，但未公开具体成绩、数量或成功率。</t>
         </is>
       </c>
+      <c r="L129" s="10" t="inlineStr"/>
+      <c r="M129" s="10" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
@@ -11760,6 +12028,8 @@
           <t>正文“nearly every challenge”不等于严格100% pass@10，未录入未经精确披露的pass@10。</t>
         </is>
       </c>
+      <c r="L130" s="10" t="inlineStr"/>
+      <c r="M130" s="10" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
@@ -11813,6 +12083,8 @@
           <t>后续Opus4.8卡报告73.1%；本条保留原卡两位小数图示值。</t>
         </is>
       </c>
+      <c r="L131" s="10" t="inlineStr"/>
+      <c r="M131" s="10" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
@@ -11866,6 +12138,8 @@
           <t>堆叠柱顶45.2%为完整+部分；后续4.8卡重跑35.2%，不覆盖此值。</t>
         </is>
       </c>
+      <c r="L132" s="10" t="inlineStr"/>
+      <c r="M132" s="10" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
@@ -11919,6 +12193,8 @@
           <t>原卡正文明确每变体3 trials，原表5 trials不符；图示值0.46为防护开启，不与无防护合并。</t>
         </is>
       </c>
+      <c r="L133" s="10" t="inlineStr"/>
+      <c r="M133" s="10" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
@@ -11972,6 +12248,8 @@
           <t>来源内部冲突：T3目标漏洞正文1.0%，图示0.9%；保留两者并明确标注。</t>
         </is>
       </c>
+      <c r="L134" s="10" t="inlineStr"/>
+      <c r="M134" s="10" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
@@ -12021,6 +12299,8 @@
         </is>
       </c>
       <c r="K135" s="10" t="inlineStr"/>
+      <c r="L135" s="10" t="inlineStr"/>
+      <c r="M135" s="10" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
@@ -12074,6 +12354,8 @@
           <t>旧harness；为分级结果，非统一成功率。</t>
         </is>
       </c>
+      <c r="L136" s="10" t="inlineStr"/>
+      <c r="M136" s="10" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
@@ -12119,6 +12401,8 @@
           <t>明确未运行</t>
         </is>
       </c>
+      <c r="L137" s="10" t="inlineStr"/>
+      <c r="M137" s="10" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
@@ -12168,6 +12452,8 @@
         </is>
       </c>
       <c r="K138" s="10" t="inlineStr"/>
+      <c r="L138" s="10" t="inlineStr"/>
+      <c r="M138" s="10" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="10" t="inlineStr">
@@ -12221,6 +12507,8 @@
           <t>不可和新Binary Exploitation Benchmark的66次劫持混合。</t>
         </is>
       </c>
+      <c r="L139" s="10" t="inlineStr"/>
+      <c r="M139" s="10" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="10" t="inlineStr">
@@ -12274,6 +12562,8 @@
           <t>218包括131次完整利用，非额外218次部分利用。</t>
         </is>
       </c>
+      <c r="L140" s="10" t="inlineStr"/>
+      <c r="M140" s="10" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="10" t="inlineStr">
@@ -12327,6 +12617,8 @@
           <t>不可与后续10场景53.0%重跑结果合并。</t>
         </is>
       </c>
+      <c r="L141" s="10" t="inlineStr"/>
+      <c r="M141" s="10" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="10" t="inlineStr">
@@ -12380,6 +12672,8 @@
           <t>图中数字为正确使用指定漏洞的利用数。</t>
         </is>
       </c>
+      <c r="L142" s="10" t="inlineStr"/>
+      <c r="M142" s="10" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="10" t="inlineStr">
@@ -12433,6 +12727,8 @@
           <t>UK AISI外部早期快照，不等同最终生产部署条件。</t>
         </is>
       </c>
+      <c r="L143" s="10" t="inlineStr"/>
+      <c r="M143" s="10" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="10" t="inlineStr">
@@ -12482,6 +12778,8 @@
         </is>
       </c>
       <c r="K144" s="10" t="inlineStr"/>
+      <c r="L144" s="10" t="inlineStr"/>
+      <c r="M144" s="10" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="10" t="inlineStr">
@@ -12531,6 +12829,8 @@
         </is>
       </c>
       <c r="K145" s="10" t="inlineStr"/>
+      <c r="L145" s="10" t="inlineStr"/>
+      <c r="M145" s="10" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="10" t="inlineStr">
@@ -12580,6 +12880,8 @@
         </is>
       </c>
       <c r="K146" s="10" t="inlineStr"/>
+      <c r="L146" s="10" t="inlineStr"/>
+      <c r="M146" s="10" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="10" t="inlineStr">
@@ -12629,6 +12931,8 @@
         </is>
       </c>
       <c r="K147" s="10" t="inlineStr"/>
+      <c r="L147" s="10" t="inlineStr"/>
+      <c r="M147" s="10" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="10" t="inlineStr">
@@ -12686,6 +12990,8 @@
           <t>网安防护关闭，escape classifiers及其他安全措施保持开启。</t>
         </is>
       </c>
+      <c r="L148" s="10" t="inlineStr"/>
+      <c r="M148" s="10" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="10" t="inlineStr">
@@ -12739,6 +13045,8 @@
         </is>
       </c>
       <c r="K149" s="10" t="inlineStr"/>
+      <c r="L149" s="10" t="inlineStr"/>
+      <c r="M149" s="10" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="10" t="inlineStr">
@@ -12796,6 +13104,8 @@
           <t>新harness重跑结果，不可与旧OSS-Fuzz直接比较。</t>
         </is>
       </c>
+      <c r="L150" s="10" t="inlineStr"/>
+      <c r="M150" s="10" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="10" t="inlineStr">
@@ -12849,6 +13159,8 @@
         </is>
       </c>
       <c r="K151" s="10" t="inlineStr"/>
+      <c r="L151" s="10" t="inlineStr"/>
+      <c r="M151" s="10" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="10" t="inlineStr">
@@ -12906,6 +13218,8 @@
           <t>网安防护关闭，escape classifiers保持开启；未披露plain均值，不能从合计ACE推算。</t>
         </is>
       </c>
+      <c r="L152" s="10" t="inlineStr"/>
+      <c r="M152" s="10" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="10" t="inlineStr">
@@ -12959,6 +13273,8 @@
         </is>
       </c>
       <c r="K153" s="10" t="inlineStr"/>
+      <c r="L153" s="10" t="inlineStr"/>
+      <c r="M153" s="10" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="10" t="inlineStr">
@@ -13016,6 +13332,8 @@
           <t>新harness重跑，不和旧OSS-Fuzz比较。</t>
         </is>
       </c>
+      <c r="L154" s="10" t="inlineStr"/>
+      <c r="M154" s="10" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="10" t="inlineStr">
@@ -13069,6 +13387,8 @@
           <t>ASLR/stack canaries/KASLR关闭；V8 sandbox除sandbox-escape任务外关闭；kernel保留SMEP/SMAP。</t>
         </is>
       </c>
+      <c r="L155" s="10" t="inlineStr"/>
+      <c r="M155" s="10" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="10" t="inlineStr">
@@ -13122,6 +13442,8 @@
         </is>
       </c>
       <c r="K156" s="10" t="inlineStr"/>
+      <c r="L156" s="10" t="inlineStr"/>
+      <c r="M156" s="10" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="10" t="inlineStr">
@@ -13179,6 +13501,8 @@
           <t>报告说明为与发布模型能力相近的预发布快照。</t>
         </is>
       </c>
+      <c r="L157" s="10" t="inlineStr"/>
+      <c r="M157" s="10" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="10" t="inlineStr">
@@ -13232,6 +13556,8 @@
         </is>
       </c>
       <c r="K158" s="10" t="inlineStr"/>
+      <c r="L158" s="10" t="inlineStr"/>
+      <c r="M158" s="10" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="10" t="inlineStr">
@@ -13285,6 +13611,8 @@
           <t>ASLR/stack canaries/KASLR关闭；V8 sandbox除sandbox-escape任务外关闭；kernel保留SMEP/SMAP。</t>
         </is>
       </c>
+      <c r="L159" s="10" t="inlineStr"/>
+      <c r="M159" s="10" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="10" t="inlineStr">
@@ -13330,6 +13658,8 @@
           <t>停止报告</t>
         </is>
       </c>
+      <c r="L160" s="10" t="inlineStr"/>
+      <c r="M160" s="10" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="10" t="inlineStr">
@@ -13379,6 +13709,8 @@
         </is>
       </c>
       <c r="K161" s="10" t="inlineStr"/>
+      <c r="L161" s="10" t="inlineStr"/>
+      <c r="M161" s="10" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="10" t="inlineStr">
@@ -13432,6 +13764,8 @@
           <t>后续卡披露83.1%，此条保留原卡0.83。</t>
         </is>
       </c>
+      <c r="L162" s="10" t="inlineStr"/>
+      <c r="M162" s="10" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="10" t="inlineStr">
@@ -13485,6 +13819,8 @@
           <t>堆叠柱顶为至少部分控制总和；后续重跑结果不同，保留本报告数值。</t>
         </is>
       </c>
+      <c r="L163" s="10" t="inlineStr"/>
+      <c r="M163" s="10" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="10" t="inlineStr">
@@ -13534,6 +13870,8 @@
           <t>仅定性披露企业网络靶场通关、OT靶场未通关及现代补丁沙箱未发现新利用；未公开精确成功次数/率。</t>
         </is>
       </c>
+      <c r="L164" s="10" t="inlineStr"/>
+      <c r="M164" s="10" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="10" t="inlineStr">
@@ -13587,6 +13925,8 @@
           <t>后续官方报告补测；后续共用卡补测，非Mythos Preview原始卡。</t>
         </is>
       </c>
+      <c r="L165" s="10" t="inlineStr"/>
+      <c r="M165" s="10" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="10" t="inlineStr">
@@ -13640,6 +13980,8 @@
           <t>后续官方报告补测</t>
         </is>
       </c>
+      <c r="L166" s="10" t="inlineStr"/>
+      <c r="M166" s="10" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="10" t="inlineStr">
@@ -13693,6 +14035,8 @@
           <t>该报告写plain超过半数环境达ACE，未给两臂合计精确ACE数；不引入后续重跑132。所有数值只归Mythos 5，非Fable 5。</t>
         </is>
       </c>
+      <c r="L167" s="10" t="inlineStr"/>
+      <c r="M167" s="10" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="10" t="inlineStr">
@@ -13746,6 +14090,8 @@
           <t>Mythos 5防护关闭；非Fable生产配置。</t>
         </is>
       </c>
+      <c r="L168" s="10" t="inlineStr"/>
+      <c r="M168" s="10" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="10" t="inlineStr">
@@ -13799,6 +14145,8 @@
           <t>Mythos 5防护关闭；非Fable生产配置。</t>
         </is>
       </c>
+      <c r="L169" s="10" t="inlineStr"/>
+      <c r="M169" s="10" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="10" t="inlineStr">
@@ -13852,6 +14200,8 @@
           <t>Mythos 5防护关闭；非Fable生产配置。</t>
         </is>
       </c>
+      <c r="L170" s="10" t="inlineStr"/>
+      <c r="M170" s="10" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="10" t="inlineStr">
@@ -13905,6 +14255,8 @@
           <t>外部UK AISI早期checkpoint；不是Fable生产配置。</t>
         </is>
       </c>
+      <c r="L171" s="10" t="inlineStr"/>
+      <c r="M171" s="10" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="10" t="inlineStr">
@@ -13950,6 +14302,8 @@
           <t>明确未运行</t>
         </is>
       </c>
+      <c r="L172" s="10" t="inlineStr"/>
+      <c r="M172" s="10" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="10" t="inlineStr">
@@ -13995,6 +14349,8 @@
           <t>不得归属给Fable生产配置</t>
         </is>
       </c>
+      <c r="L173" s="10" t="inlineStr"/>
+      <c r="M173" s="10" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="10" t="inlineStr">
@@ -14040,6 +14396,8 @@
           <t>不得归属给Fable生产配置</t>
         </is>
       </c>
+      <c r="L174" s="10" t="inlineStr"/>
+      <c r="M174" s="10" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="10" t="inlineStr">
@@ -14085,6 +14443,8 @@
           <t>不得归属给Fable生产配置</t>
         </is>
       </c>
+      <c r="L175" s="10" t="inlineStr"/>
+      <c r="M175" s="10" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="10" t="inlineStr">
@@ -14130,6 +14490,8 @@
           <t>不得归属给Fable生产配置</t>
         </is>
       </c>
+      <c r="L176" s="10" t="inlineStr"/>
+      <c r="M176" s="10" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="10" t="inlineStr">
@@ -14175,6 +14537,8 @@
           <t>不得归属给Fable生产配置</t>
         </is>
       </c>
+      <c r="L177" s="10" t="inlineStr"/>
+      <c r="M177" s="10" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="10" t="inlineStr">
@@ -14220,6 +14584,8 @@
           <t>不得归属给Fable生产配置</t>
         </is>
       </c>
+      <c r="L178" s="10" t="inlineStr"/>
+      <c r="M178" s="10" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="10" t="inlineStr">
@@ -14265,6 +14631,8 @@
           <t>不得归属给Fable生产配置</t>
         </is>
       </c>
+      <c r="L179" s="10" t="inlineStr"/>
+      <c r="M179" s="10" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="10" t="inlineStr">
@@ -14310,6 +14678,8 @@
           <t>不得归属给Fable生产配置</t>
         </is>
       </c>
+      <c r="L180" s="10" t="inlineStr"/>
+      <c r="M180" s="10" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="10" t="inlineStr">
@@ -14363,6 +14733,8 @@
           <t>本卡222/410；后续卡重跑221，不覆盖此条。Mythos 5.1防护关闭，非Fable 5.1。</t>
         </is>
       </c>
+      <c r="L181" s="10" t="inlineStr"/>
+      <c r="M181" s="10" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="10" t="inlineStr">
@@ -14412,6 +14784,8 @@
         </is>
       </c>
       <c r="K182" s="10" t="inlineStr"/>
+      <c r="L182" s="10" t="inlineStr"/>
+      <c r="M182" s="10" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="10" t="inlineStr">
@@ -14461,6 +14835,8 @@
         </is>
       </c>
       <c r="K183" s="10" t="inlineStr"/>
+      <c r="L183" s="10" t="inlineStr"/>
+      <c r="M183" s="10" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="10" t="inlineStr">
@@ -14514,6 +14890,8 @@
           <t>Mythos 5.1防护关闭；非Fable 5.1生产配置。</t>
         </is>
       </c>
+      <c r="L184" s="10" t="inlineStr"/>
+      <c r="M184" s="10" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="10" t="inlineStr">
@@ -14559,6 +14937,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L185" s="10" t="inlineStr"/>
+      <c r="M185" s="10" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="10" t="inlineStr">
@@ -14604,6 +14984,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L186" s="10" t="inlineStr"/>
+      <c r="M186" s="10" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="10" t="inlineStr">
@@ -14657,6 +15039,8 @@
           <t>无公开数值成绩；3.1 Pro与Deep Think均进行了额外网安测试；报告称计入推理成本Deep Think更差，不能继承其他版本分数。</t>
         </is>
       </c>
+      <c r="L187" s="10" t="inlineStr"/>
+      <c r="M187" s="10" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="10" t="inlineStr">
@@ -14702,6 +15086,8 @@
           <t>仅方法引用</t>
         </is>
       </c>
+      <c r="L188" s="10" t="inlineStr"/>
+      <c r="M188" s="10" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="10" t="inlineStr">
@@ -14747,6 +15133,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L189" s="10" t="inlineStr"/>
+      <c r="M189" s="10" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="10" t="inlineStr">
@@ -14792,6 +15180,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L190" s="10" t="inlineStr"/>
+      <c r="M190" s="10" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="10" t="inlineStr">
@@ -14837,6 +15227,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L191" s="10" t="inlineStr"/>
+      <c r="M191" s="10" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="10" t="inlineStr">
@@ -14890,6 +15282,8 @@
           <t>只披露阈值判断，没有具名题集、原始分数或成功率。</t>
         </is>
       </c>
+      <c r="L192" s="10" t="inlineStr"/>
+      <c r="M192" s="10" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="10" t="inlineStr">
@@ -14943,6 +15337,8 @@
           <t>只披露阈值判断，没有具名题集、原始分数或成功率。</t>
         </is>
       </c>
+      <c r="L193" s="10" t="inlineStr"/>
+      <c r="M193" s="10" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="10" t="inlineStr">
@@ -14996,6 +15392,8 @@
           <t>CodeMender多智能体组合报告；整页视觉核对无分数图表。</t>
         </is>
       </c>
+      <c r="L194" s="10" t="inlineStr"/>
+      <c r="M194" s="10" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="10" t="inlineStr">
@@ -15049,6 +15447,8 @@
           <t>使用网安、软件工程和综合能力代理评测预测uplift，未公开具名代理原始数值；能力评估未运行Key Skills，不可与防护设置Key Skills混淆。</t>
         </is>
       </c>
+      <c r="L195" s="10" t="inlineStr"/>
+      <c r="M195" s="10" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="10" t="inlineStr">
@@ -15094,6 +15494,8 @@
           <t>明确未运行</t>
         </is>
       </c>
+      <c r="L196" s="10" t="inlineStr"/>
+      <c r="M196" s="10" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="10" t="inlineStr">
@@ -15151,6 +15553,8 @@
           <t>防护拒答率；不是任务成功率。</t>
         </is>
       </c>
+      <c r="L197" s="10" t="inlineStr"/>
+      <c r="M197" s="10" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="10" t="inlineStr">
@@ -15204,6 +15608,8 @@
           <t>视觉读取图5明确数字；与前代使用同图对比，但只提取目标模型。</t>
         </is>
       </c>
+      <c r="L198" s="10" t="inlineStr"/>
+      <c r="M198" s="10" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="10" t="inlineStr">
@@ -15257,6 +15663,8 @@
           <t>越狱攻击成功率，越低越好；图示95% Jeffreys Beta置信区间。</t>
         </is>
       </c>
+      <c r="L199" s="10" t="inlineStr"/>
+      <c r="M199" s="10" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="10" t="inlineStr">
@@ -15310,6 +15718,8 @@
           <t>未根据柱高猜测QSR，也未填0；OSR为图中明确标注值。攻击成功率，越低越好。</t>
         </is>
       </c>
+      <c r="L200" s="10" t="inlineStr"/>
+      <c r="M200" s="10" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="10" t="inlineStr">
@@ -15363,6 +15773,8 @@
           <t>28项cyber tasks，Shade自动红队，高thinking；攻击成功率，越低越好。</t>
         </is>
       </c>
+      <c r="L201" s="10" t="inlineStr"/>
+      <c r="M201" s="10" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="10" t="inlineStr">
@@ -15416,6 +15828,8 @@
           <t>后续报告补测／历史对比披露；非原始发布页披露。原发布页仅定性描述；数值由后续Gemini4安全报告图6.9补录，不表示原发布时已披露。k=1、k=10无数字标注未估读；越低越好。</t>
         </is>
       </c>
+      <c r="L202" s="10" t="inlineStr"/>
+      <c r="M202" s="10" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="10" t="inlineStr">
@@ -15469,6 +15883,8 @@
           <t>后续报告补测／历史对比披露；非原始发布页披露。原发布页仅定性描述；数值由后续Gemini4安全报告图6.9补录，不表示原发布时已披露。k=1、k=10无数字标注未估读；越低越好。</t>
         </is>
       </c>
+      <c r="L203" s="10" t="inlineStr"/>
+      <c r="M203" s="10" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="10" t="inlineStr">
@@ -15522,6 +15938,8 @@
           <t>原发布页文本和视觉核对均无该评测分数。</t>
         </is>
       </c>
+      <c r="L204" s="10" t="inlineStr"/>
+      <c r="M204" s="10" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="10" t="inlineStr">
@@ -15579,6 +15997,8 @@
           <t>漏洞修复能力；不继承对比模型47.8%。</t>
         </is>
       </c>
+      <c r="L205" s="10" t="inlineStr"/>
+      <c r="M205" s="10" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="10" t="inlineStr">
@@ -15636,6 +16056,8 @@
           <t>原文为严格大于70%，不写作精确70%。</t>
         </is>
       </c>
+      <c r="L206" s="10" t="inlineStr"/>
+      <c r="M206" s="10" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="10" t="inlineStr">
@@ -15693,6 +16115,8 @@
           <t>数量比值；未披露绝对补丁数或成功率。</t>
         </is>
       </c>
+      <c r="L207" s="10" t="inlineStr"/>
+      <c r="M207" s="10" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="10" t="inlineStr">
@@ -15750,6 +16174,8 @@
           <t>原文未说明百分数是相对百分比还是百分点，保留原文表述，不擅自改为pp。</t>
         </is>
       </c>
+      <c r="L208" s="10" t="inlineStr"/>
+      <c r="M208" s="10" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="10" t="inlineStr">
@@ -15807,6 +16233,8 @@
           <t>Model C最终候选，不加模型外防护；两个挑战通过非预期解法解决，原始成功率与uplift可能高估预期任务表现。图中pass@k曲线无逐点数字，未估读。</t>
         </is>
       </c>
+      <c r="L209" s="10" t="inlineStr"/>
+      <c r="M209" s="10" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="10" t="inlineStr">
@@ -15864,6 +16292,8 @@
           <t>41个挑战，每个16项能力；不是挑战级成功率，也不是pass@1。</t>
         </is>
       </c>
+      <c r="L210" s="10" t="inlineStr"/>
+      <c r="M210" s="10" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="10" t="inlineStr">
@@ -15921,6 +16351,8 @@
           <t>真实代码库开放式漏洞发现；不同于20-language benchmark。</t>
         </is>
       </c>
+      <c r="L211" s="10" t="inlineStr"/>
+      <c r="M211" s="10" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="10" t="inlineStr">
@@ -15974,6 +16406,8 @@
         </is>
       </c>
       <c r="K212" s="10" t="inlineStr"/>
+      <c r="L212" s="10" t="inlineStr"/>
+      <c r="M212" s="10" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="10" t="inlineStr">
@@ -16031,6 +16465,8 @@
           <t>所有既有功能和回归测试需通过；分数为120任务平均成功率，不是四次取最好。</t>
         </is>
       </c>
+      <c r="L213" s="10" t="inlineStr"/>
+      <c r="M213" s="10" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="10" t="inlineStr">
@@ -16084,6 +16520,8 @@
           <t>本段将两个防护评测合并叙述，不单独推断每个题集能力成功率。</t>
         </is>
       </c>
+      <c r="L214" s="10" t="inlineStr"/>
+      <c r="M214" s="10" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="10" t="inlineStr">
@@ -16137,6 +16575,8 @@
           <t>防护效果和良性使用代价分别保留，不把近100%覆盖写成精确100%。</t>
         </is>
       </c>
+      <c r="L215" s="10" t="inlineStr"/>
+      <c r="M215" s="10" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="10" t="inlineStr">
@@ -16190,6 +16630,8 @@
           <t>正文说close to 0%，图中明确&lt;1%，保留上界而不填精确0%。攻击成功率，越低越好。</t>
         </is>
       </c>
+      <c r="L216" s="10" t="inlineStr"/>
+      <c r="M216" s="10" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="10" t="inlineStr">
@@ -16243,6 +16685,8 @@
           <t>正文和图表一致；攻击成功率，越低越好。</t>
         </is>
       </c>
+      <c r="L217" s="10" t="inlineStr"/>
+      <c r="M217" s="10" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="10" t="inlineStr">
@@ -16296,6 +16740,8 @@
           <t>25项cyber任务，Shade自动红队，高thinking；原文62页确认QSR10%。攻击成功率，越低越好。</t>
         </is>
       </c>
+      <c r="L218" s="10" t="inlineStr"/>
+      <c r="M218" s="10" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="10" t="inlineStr">
@@ -16349,6 +16795,8 @@
           <t>间接提示注入鲁棒性，越低越好；k=1/k=10无精确标注未估读。</t>
         </is>
       </c>
+      <c r="L219" s="10" t="inlineStr"/>
+      <c r="M219" s="10" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="10" t="inlineStr">
@@ -16398,6 +16846,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L220" s="10" t="inlineStr"/>
+      <c r="M220" s="10" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="10" t="inlineStr">
@@ -16447,6 +16897,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L221" s="10" t="inlineStr"/>
+      <c r="M221" s="10" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="10" t="inlineStr">
@@ -16496,6 +16948,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L222" s="10" t="inlineStr"/>
+      <c r="M222" s="10" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="10" t="inlineStr">
@@ -16545,6 +16999,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L223" s="10" t="inlineStr"/>
+      <c r="M223" s="10" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="10" t="inlineStr">
@@ -16594,6 +17050,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L224" s="10" t="inlineStr"/>
+      <c r="M224" s="10" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="10" t="inlineStr">
@@ -16643,6 +17101,8 @@
           <t>已渲染查看；报告给出该模型曲线，未标注精确数据点，不估读。不同预算/2h与6h上限不得合为一个百分比。</t>
         </is>
       </c>
+      <c r="L225" s="10" t="inlineStr"/>
+      <c r="M225" s="10" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="10" t="inlineStr">
@@ -16696,6 +17156,8 @@
           <t>CyberGym用作越狱迁移/能力退化及端到端防护测试，四种配置单列，不和公开能力排行榜混用。</t>
         </is>
       </c>
+      <c r="L226" s="10" t="inlineStr"/>
+      <c r="M226" s="10" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="10" t="inlineStr">
@@ -16749,6 +17211,8 @@
           <t>CyberGym用作越狱迁移/能力退化及端到端防护测试，四种配置单列，不和公开能力排行榜混用。</t>
         </is>
       </c>
+      <c r="L227" s="10" t="inlineStr"/>
+      <c r="M227" s="10" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="10" t="inlineStr">
@@ -16802,6 +17266,8 @@
           <t>后续官方报告补测；堆叠柱顶为至少部分控制总和；后续重跑结果不同，保留本报告数值。；自查移除top 2条件的完整利用柱段无精确标注，未将未见柱段推断成0%；其余百分数均为图上明确标签。</t>
         </is>
       </c>
+      <c r="L228" s="10" t="inlineStr"/>
+      <c r="M228" s="10" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
@@ -16855,6 +17321,8 @@
           <t>后续官方报告补测；堆叠柱顶为至少部分控制总和；后续重跑结果不同，保留本报告数值。；自查标准条件的完整利用柱段无精确标注，未将未见柱段推断成0%；其余百分数均为图上明确标签。</t>
         </is>
       </c>
+      <c r="L229" s="10" t="inlineStr"/>
+      <c r="M229" s="10" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
@@ -16908,6 +17376,8 @@
           <t>后续官方报告补测</t>
         </is>
       </c>
+      <c r="L230" s="10" t="inlineStr"/>
+      <c r="M230" s="10" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="10" t="inlineStr">
@@ -16961,6 +17431,8 @@
           <t>后续官方报告补测</t>
         </is>
       </c>
+      <c r="L231" s="10" t="inlineStr"/>
+      <c r="M231" s="10" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="10" t="inlineStr">
@@ -17014,6 +17486,8 @@
           <t>后续官方报告补测；后续卡补测；旧harness。</t>
         </is>
       </c>
+      <c r="L232" s="10" t="inlineStr"/>
+      <c r="M232" s="10" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="10" t="inlineStr">
@@ -17071,6 +17545,8 @@
           <t>后续报告，不是Mythos5.1原始卡逐项披露</t>
         </is>
       </c>
+      <c r="L233" s="10" t="inlineStr"/>
+      <c r="M233" s="10" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="10" t="inlineStr">
@@ -17128,6 +17604,8 @@
           <t>与Opus5卡9场景配置区分；与Opus5原卡9场景配置的3.3%不同。</t>
         </is>
       </c>
+      <c r="L234" s="10" t="inlineStr"/>
+      <c r="M234" s="10" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="10" t="inlineStr">
@@ -17181,6 +17659,8 @@
           <t>后续重跑且更名；新harness重跑，不能和原始OSS-Fuzz旧harness成绩直接比较。</t>
         </is>
       </c>
+      <c r="L235" s="10" t="inlineStr"/>
+      <c r="M235" s="10" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="10" t="inlineStr">
@@ -17234,6 +17714,8 @@
           <t>后续重跑且更名；新harness重跑，不能和原始OSS-Fuzz旧harness成绩直接比较。</t>
         </is>
       </c>
+      <c r="L236" s="10" t="inlineStr"/>
+      <c r="M236" s="10" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="10" t="inlineStr">
@@ -17287,6 +17769,8 @@
           <t>后续重跑且更名；新harness重跑，不能和原始OSS-Fuzz旧harness成绩直接比较。</t>
         </is>
       </c>
+      <c r="L237" s="10" t="inlineStr"/>
+      <c r="M237" s="10" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="10" t="inlineStr">
@@ -17340,6 +17824,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L238" s="10" t="inlineStr"/>
+      <c r="M238" s="10" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="10" t="inlineStr">
@@ -17393,6 +17879,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L239" s="10" t="inlineStr"/>
+      <c r="M239" s="10" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="10" t="inlineStr">
@@ -17447,6 +17935,8 @@
           <t>已人工读取官方基准表图片；原文goal.txt漏列。；原始图表：docs/DeepSeek/v4_260821_benchmark_en.png</t>
         </is>
       </c>
+      <c r="L240" s="10" t="inlineStr"/>
+      <c r="M240" s="10" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="10" t="inlineStr">
@@ -17501,6 +17991,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L241" s="10" t="inlineStr"/>
+      <c r="M241" s="10" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="10" t="inlineStr">
@@ -17555,6 +18047,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L242" s="10" t="inlineStr"/>
+      <c r="M242" s="10" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="10" t="inlineStr">
@@ -17609,6 +18103,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L243" s="10" t="inlineStr"/>
+      <c r="M243" s="10" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="10" t="inlineStr">
@@ -17662,6 +18158,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L244" s="10" t="inlineStr"/>
+      <c r="M244" s="10" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="10" t="inlineStr">
@@ -17715,6 +18213,8 @@
           <t>后续报告比较值；保留首发43.2，不覆盖原值。</t>
         </is>
       </c>
+      <c r="L245" s="10" t="inlineStr"/>
+      <c r="M245" s="10" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="10" t="inlineStr">
@@ -17768,6 +18268,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L246" s="10" t="inlineStr"/>
+      <c r="M246" s="10" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="10" t="inlineStr">
@@ -17821,6 +18323,8 @@
           <t>后续同厂报告补测</t>
         </is>
       </c>
+      <c r="L247" s="10" t="inlineStr"/>
+      <c r="M247" s="10" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="10" t="inlineStr">
@@ -17874,6 +18378,8 @@
           <t>后续同厂报告补测</t>
         </is>
       </c>
+      <c r="L248" s="10" t="inlineStr"/>
+      <c r="M248" s="10" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="10" t="inlineStr">
@@ -17927,6 +18433,8 @@
           <t>后续同厂报告补测</t>
         </is>
       </c>
+      <c r="L249" s="10" t="inlineStr"/>
+      <c r="M249" s="10" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="10" t="inlineStr">
@@ -17980,6 +18488,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L250" s="10" t="inlineStr"/>
+      <c r="M250" s="10" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="10" t="inlineStr">
@@ -18033,6 +18543,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L251" s="10" t="inlineStr"/>
+      <c r="M251" s="10" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="10" t="inlineStr">
@@ -18086,6 +18598,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L252" s="10" t="inlineStr"/>
+      <c r="M252" s="10" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" s="10" t="inlineStr">
@@ -18139,6 +18653,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L253" s="10" t="inlineStr"/>
+      <c r="M253" s="10" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="10" t="inlineStr">
@@ -18192,6 +18708,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L254" s="10" t="inlineStr"/>
+      <c r="M254" s="10" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" s="10" t="inlineStr">
@@ -18237,6 +18755,8 @@
           <t>模型覆盖待核对</t>
         </is>
       </c>
+      <c r="L255" s="10" t="inlineStr"/>
+      <c r="M255" s="10" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="10" t="inlineStr">
@@ -18290,6 +18810,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L256" s="10" t="inlineStr"/>
+      <c r="M256" s="10" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="10" t="inlineStr">
@@ -18343,6 +18865,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L257" s="10" t="inlineStr"/>
+      <c r="M257" s="10" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" s="10" t="inlineStr">
@@ -18396,6 +18920,8 @@
           <t>依据本地归档官方报告逐项复核；比例按原指标换算，不与不同配置合并。</t>
         </is>
       </c>
+      <c r="L258" s="10" t="inlineStr"/>
+      <c r="M258" s="10" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" s="10" t="inlineStr">
@@ -18450,6 +18976,8 @@
           <t>后续官方报告补测；已人工核对官方图片；原表漏列。证据图片：docs/Tencent/hy4-benchmark-appendix.jpg</t>
         </is>
       </c>
+      <c r="L259" s="10" t="inlineStr"/>
+      <c r="M259" s="10" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="10" t="inlineStr">
@@ -18504,6 +19032,8 @@
           <t>已人工核对官方图片；原表漏列。证据图片：docs/Tencent/hy4-benchmark-appendix.jpg</t>
         </is>
       </c>
+      <c r="L260" s="10" t="inlineStr"/>
+      <c r="M260" s="10" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" s="10" t="inlineStr">
@@ -18549,6 +19079,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L261" s="10" t="inlineStr"/>
+      <c r="M261" s="10" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="10" t="inlineStr">
@@ -18594,6 +19126,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L262" s="10" t="inlineStr"/>
+      <c r="M262" s="10" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="10" t="inlineStr">
@@ -18639,6 +19173,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L263" s="10" t="inlineStr"/>
+      <c r="M263" s="10" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="10" t="inlineStr">
@@ -18684,6 +19220,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L264" s="10" t="inlineStr"/>
+      <c r="M264" s="10" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="10" t="inlineStr">
@@ -18729,6 +19267,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L265" s="10" t="inlineStr"/>
+      <c r="M265" s="10" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="10" t="inlineStr">
@@ -18774,6 +19314,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L266" s="10" t="inlineStr"/>
+      <c r="M266" s="10" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="10" t="inlineStr">
@@ -18819,6 +19361,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L267" s="10" t="inlineStr"/>
+      <c r="M267" s="10" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="10" t="inlineStr">
@@ -18864,6 +19408,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L268" s="10" t="inlineStr"/>
+      <c r="M268" s="10" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="10" t="inlineStr">
@@ -18909,6 +19455,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L269" s="10" t="inlineStr"/>
+      <c r="M269" s="10" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="10" t="inlineStr">
@@ -18954,6 +19502,8 @@
           <t>同模型服务档位</t>
         </is>
       </c>
+      <c r="L270" s="10" t="inlineStr"/>
+      <c r="M270" s="10" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="10" t="inlineStr">
@@ -18999,6 +19549,8 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L271" s="10" t="inlineStr"/>
+      <c r="M271" s="10" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="10" t="inlineStr">
@@ -19044,9 +19596,841 @@
           <t>未披露具名项目</t>
         </is>
       </c>
+      <c r="L272" s="10" t="inlineStr"/>
+      <c r="M272" s="10" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0269</t>
+        </is>
+      </c>
+      <c r="B273" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K2.5</t>
+        </is>
+      </c>
+      <c r="C273" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D273" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E273" s="10" t="inlineStr">
+        <is>
+          <t>41.3%</t>
+        </is>
+      </c>
+      <c r="F273" s="10" t="inlineStr"/>
+      <c r="G273" s="10" t="inlineStr">
+        <is>
+          <t>table/text</t>
+        </is>
+      </c>
+      <c r="H273" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-5.pdf p.11-12,26</t>
+        </is>
+      </c>
+      <c r="I273" s="10" t="inlineStr">
+        <is>
+          <t>Table 4: CyberGym 41.3. Appendix E.5: difficulty level 1; coding task results averaged over 5 independent runs (Avg@5).</t>
+        </is>
+      </c>
+      <c r="J273" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "Avg@5成功率", "value": 41.3, "unit": "percent", "configuration": "Moonshot技术报告；CyberGym difficulty level 1；编程任务按5次独立运行取平均（Avg@5），不标为pass@1。"}]</t>
+        </is>
+      </c>
+      <c r="K273" s="10" t="inlineStr">
+        <is>
+          <t>41.3按原表百分制保存；保留Avg@5和difficulty level 1，不与其他harness的pass@1合并。 技术报告提交日为2月2日，不称为1月27日首发成绩。</t>
+        </is>
+      </c>
+      <c r="L273" s="10" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="M273" s="10" t="inlineStr">
+        <is>
+          <t>vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0270</t>
+        </is>
+      </c>
+      <c r="B274" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K2.6</t>
+        </is>
+      </c>
+      <c r="C274" s="10" t="inlineStr">
+        <is>
+          <t>CyberBench v1</t>
+        </is>
+      </c>
+      <c r="D274" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E274" s="10" t="inlineStr">
+        <is>
+          <t>74.35%</t>
+        </is>
+      </c>
+      <c r="F274" s="10" t="inlineStr"/>
+      <c r="G274" s="10" t="inlineStr">
+        <is>
+          <t>archived_web</t>
+        </is>
+      </c>
+      <c r="H274" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/vals-cyberbench-v1.mhtml Overall leaderboard / Methodology</t>
+        </is>
+      </c>
+      <c r="I274" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 — Overall Accuracy 74.35%. v1 results archived; superseded by v1.1.</t>
+        </is>
+      </c>
+      <c r="J274" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "准确率", "value": 74.35, "unit": "percent", "configuration": "Vals AI独立机构评测；2026-09-16归档v1；60题PoC与原Patch设置；Overall accuracy；不得与v1.1直接比较。"}]</t>
+        </is>
+      </c>
+      <c r="K274" s="10" t="inlineStr"/>
+      <c r="L274" s="10" t="inlineStr">
+        <is>
+          <t>Vals AI</t>
+        </is>
+      </c>
+      <c r="M274" s="10" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0271</t>
+        </is>
+      </c>
+      <c r="B275" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C275" s="10" t="inlineStr">
+        <is>
+          <t>CyberBench v1</t>
+        </is>
+      </c>
+      <c r="D275" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E275" s="10" t="inlineStr">
+        <is>
+          <t>79.03%</t>
+        </is>
+      </c>
+      <c r="F275" s="10" t="inlineStr"/>
+      <c r="G275" s="10" t="inlineStr">
+        <is>
+          <t>archived_web</t>
+        </is>
+      </c>
+      <c r="H275" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/vals-cyberbench-v1.mhtml Overall leaderboard / Methodology</t>
+        </is>
+      </c>
+      <c r="I275" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3 — Overall Accuracy 79.03%. v1 results archived; superseded by v1.1.</t>
+        </is>
+      </c>
+      <c r="J275" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "准确率", "value": 79.03, "unit": "percent", "configuration": "Vals AI独立机构评测；2026-09-16归档v1；60题PoC与原Patch设置；Overall accuracy；不得与v1.1直接比较。"}]</t>
+        </is>
+      </c>
+      <c r="K275" s="10" t="inlineStr"/>
+      <c r="L275" s="10" t="inlineStr">
+        <is>
+          <t>Vals AI</t>
+        </is>
+      </c>
+      <c r="M275" s="10" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0272</t>
+        </is>
+      </c>
+      <c r="B276" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C276" s="10" t="inlineStr">
+        <is>
+          <t>CyberBench v1.1</t>
+        </is>
+      </c>
+      <c r="D276" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E276" s="10" t="inlineStr">
+        <is>
+          <t>75.24%</t>
+        </is>
+      </c>
+      <c r="F276" s="10" t="inlineStr"/>
+      <c r="G276" s="10" t="inlineStr">
+        <is>
+          <t>archived_web</t>
+        </is>
+      </c>
+      <c r="H276" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/vals-cyberbench-v1-1.mhtml Overall leaderboard / Methodology</t>
+        </is>
+      </c>
+      <c r="I276" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3 — Overall Accuracy 75.24%. Rerun with offline task sandboxes, hardened clean-room grader; 60-task PoC track and 56-task Patch roster.</t>
+        </is>
+      </c>
+      <c r="J276" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "准确率", "value": 75.24, "unit": "percent", "configuration": "Vals AI独立机构评测；2026-10-12版v1.1；60题PoC、56题Patch；离线任务沙箱与加固clean-room grader；Overall accuracy；不得与v1直接比较。"}]</t>
+        </is>
+      </c>
+      <c r="K276" s="10" t="inlineStr"/>
+      <c r="L276" s="10" t="inlineStr">
+        <is>
+          <t>Vals AI</t>
+        </is>
+      </c>
+      <c r="M276" s="10" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0273</t>
+        </is>
+      </c>
+      <c r="B277" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C277" s="10" t="inlineStr">
+        <is>
+          <t>Real-world Vulnerability Discovery</t>
+        </is>
+      </c>
+      <c r="D277" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E277" s="10" t="inlineStr">
+        <is>
+          <t>16个此前未知漏洞／6项目；人工复核候选约70%确认</t>
+        </is>
+      </c>
+      <c r="F277" s="10" t="inlineStr"/>
+      <c r="G277" s="10" t="inlineStr">
+        <is>
+          <t>table/text</t>
+        </is>
+      </c>
+      <c r="H277" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k3.pdf p.30</t>
+        </is>
+      </c>
+      <c r="I277" s="10" t="inlineStr">
+        <is>
+          <t>Of the findings that underwent human review, approximately 70% were confirmed as genuine, including 16 previously unknown vulnerabilities across six projects.</t>
+        </is>
+      </c>
+      <c r="J277" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "此前未知漏洞数", "value": 16, "unit": "count", "configuration": "Moonshot K3技术报告§6.2.2 Tier 1；真实软件及内部基础设施；约70%仅指经过人工复核的候选，不是全部任务成功率；16个此前未知漏洞涉及6个项目。"}, {"label": "涉及项目数", "value": 6, "unit": "count", "configuration": "Moonshot K3技术报告§6.2.2 Tier 1；真实软件及内部基础设施；约70%仅指经过人工复核的候选，不是全部任务成功率；16个此前未知漏洞涉及6个项目。"}, {"label": "人工复核确认比例", "value": "~70", "unit": "percent", "configuration": "Moonshot K3技术报告§6.2.2 Tier 1；真实软件及内部基础设施；约70%仅指经过人工复核的候选，不是全部任务成功率；16个此前未知漏洞涉及6个项目。"}]</t>
+        </is>
+      </c>
+      <c r="K277" s="10" t="inlineStr">
+        <is>
+          <t>约70%保留为带限定字符串，不作为精确数值点绘图；候选漏洞确认率不是任务成功率。 报告包含截至7月23日的独立评估；不称为7月16日首发成绩，精确报告发表日未另核。</t>
+        </is>
+      </c>
+      <c r="L277" s="10" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="M277" s="10" t="inlineStr">
+        <is>
+          <t>vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0274</t>
+        </is>
+      </c>
+      <c r="B278" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C278" s="10" t="inlineStr">
+        <is>
+          <t>In-house exploit suite (36 tasks; Moonshot)</t>
+        </is>
+      </c>
+      <c r="D278" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E278" s="10" t="inlineStr">
+        <is>
+          <t>14/36（38.9%）；其中10题来自用户态</t>
+        </is>
+      </c>
+      <c r="F278" s="10" t="inlineStr"/>
+      <c r="G278" s="10" t="inlineStr">
+        <is>
+          <t>table/text</t>
+        </is>
+      </c>
+      <c r="H278" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k3.pdf p.30-31</t>
+        </is>
+      </c>
+      <c r="I278" s="10" t="inlineStr">
+        <is>
+          <t>Solving 14 of 36 tasks (38.9%) versus 8 of 36 (22.2%) for GLM-5.2; 10 of the 14 come from the user-space track.</t>
+        </is>
+      </c>
+      <c r="J278" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "成功率", "value": 38.9, "unit": "percent", "configuration": "Moonshot内部36题利用集；16题用户态、20题Linux内核；GLM-5.2为基线；不同加固等级，不能等同公开ExploitGym或ExploitBench。"}, {"label": "已解挑战", "value": 14, "unit": "count", "configuration": "Moonshot内部36题利用集；16题用户态、20题Linux内核；GLM-5.2为基线；不同加固等级，不能等同公开ExploitGym或ExploitBench。"}, {"label": "用户态成功任务数", "value": 10, "unit": "count", "configuration": "Moonshot内部36题利用集；16题用户态、20题Linux内核；GLM-5.2为基线；不同加固等级，不能等同公开ExploitGym或ExploitBench。"}]</t>
+        </is>
+      </c>
+      <c r="K278" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 报告包含截至7月23日的独立评估；不称为7月16日首发成绩，精确报告发表日未另核。</t>
+        </is>
+      </c>
+      <c r="L278" s="10" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="M278" s="10" t="inlineStr">
+        <is>
+          <t>vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0275</t>
+        </is>
+      </c>
+      <c r="B279" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C279" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym</t>
+        </is>
+      </c>
+      <c r="D279" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E279" s="10" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="F279" s="10" t="inlineStr"/>
+      <c r="G279" s="10" t="inlineStr">
+        <is>
+          <t>archived_web</t>
+        </is>
+      </c>
+      <c r="H279" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml Performance table / CyberGym</t>
+        </is>
+      </c>
+      <c r="I279" s="10" t="inlineStr">
+        <is>
+          <t>CyberGym row: GLM-5.3 84.5, GLM-5.2 77.2, Kimi K3 80.0.</t>
+        </is>
+      </c>
+      <c r="J279" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "目标漏洞复现", "value": 80, "unit": "percent", "configuration": "智谱GLM-5.3博客中的Kimi K3比较列；CyberGym 1507题single-run pass@1；不把GLM-5.3专属harness设置自动归给Kimi。"}]</t>
+        </is>
+      </c>
+      <c r="K279" s="10" t="inlineStr"/>
+      <c r="L279" s="10" t="inlineStr">
+        <is>
+          <t>Zhipu / GLM</t>
+        </is>
+      </c>
+      <c r="M279" s="10" t="inlineStr">
+        <is>
+          <t>cross-vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0276</t>
+        </is>
+      </c>
+      <c r="B280" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C280" s="10" t="inlineStr">
+        <is>
+          <t>ExploitGym</t>
+        </is>
+      </c>
+      <c r="D280" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E280" s="10" t="inlineStr">
+        <is>
+          <t>2h:36题；6h:70题</t>
+        </is>
+      </c>
+      <c r="F280" s="10" t="inlineStr"/>
+      <c r="G280" s="10" t="inlineStr">
+        <is>
+          <t>archived_web</t>
+        </is>
+      </c>
+      <c r="H280" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml Performance table / ExploitGym footnote</t>
+        </is>
+      </c>
+      <c r="I280" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3: ExploitGym 2h / 6h = 36 / 70. Footnote explicitly evaluates Kimi-K3 in Claude Code 2.1.207 and normalizes by 40 TPS.</t>
+        </is>
+      </c>
+      <c r="J280" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "完成任务数", "value": 36, "unit": "count", "configuration": "智谱GLM-5.3博客对Kimi K3实测；Claude Code2.1.207，max，no web，temperature=1，top_p=1，max_new_tokens=128000；869题；按40 TPS归一化API推理时间加非API开销；2h预算；数值为完成题数。"}, {"label": "完成任务数", "value": 70, "unit": "count", "configuration": "智谱GLM-5.3博客对Kimi K3实测；Claude Code2.1.207，max，no web，temperature=1，top_p=1，max_new_tokens=128000；869题；按40 TPS归一化API推理时间加非API开销；6h预算；数值为完成题数。"}]</t>
+        </is>
+      </c>
+      <c r="K280" s="10" t="inlineStr"/>
+      <c r="L280" s="10" t="inlineStr">
+        <is>
+          <t>Zhipu / GLM</t>
+        </is>
+      </c>
+      <c r="M280" s="10" t="inlineStr">
+        <is>
+          <t>cross-vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0277</t>
+        </is>
+      </c>
+      <c r="B281" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C281" s="10" t="inlineStr">
+        <is>
+          <t>ExploitBench</t>
+        </is>
+      </c>
+      <c r="D281" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E281" s="10" t="inlineStr">
+        <is>
+          <t>32.2%</t>
+        </is>
+      </c>
+      <c r="F281" s="10" t="inlineStr"/>
+      <c r="G281" s="10" t="inlineStr">
+        <is>
+          <t>archived_web</t>
+        </is>
+      </c>
+      <c r="H281" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Zhipu/glm-5-3.mhtml Performance table / ExploitBench</t>
+        </is>
+      </c>
+      <c r="I281" s="10" t="inlineStr">
+        <is>
+          <t>ExploitBench row: GLM-5.3 54.4, GLM-5.2 24.4, Kimi K3 32.2.</t>
+        </is>
+      </c>
+      <c r="J281" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "Cap%", "value": 32.2, "unit": "percent", "configuration": "智谱GLM-5.3博客中的Kimi K3比较列；ExploitBench能力覆盖32.2%；不是完整ACE成功率；与AISI的32%分别保留，不平均。"}]</t>
+        </is>
+      </c>
+      <c r="K281" s="10" t="inlineStr"/>
+      <c r="L281" s="10" t="inlineStr">
+        <is>
+          <t>Zhipu / GLM</t>
+        </is>
+      </c>
+      <c r="M281" s="10" t="inlineStr">
+        <is>
+          <t>cross-vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0278</t>
+        </is>
+      </c>
+      <c r="B282" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C282" s="10" t="inlineStr">
+        <is>
+          <t>ExploitBench</t>
+        </is>
+      </c>
+      <c r="D282" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E282" s="10" t="inlineStr">
+        <is>
+          <t>Cap 32%；完整ACE 0/41</t>
+        </is>
+      </c>
+      <c r="F282" s="10" t="inlineStr"/>
+      <c r="G282" s="10" t="inlineStr">
+        <is>
+          <t>archived_web</t>
+        </is>
+      </c>
+      <c r="H282" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/aisi-kimi-k3.mhtml Exploit Development: ExploitBench / Figures 1 and 3</t>
+        </is>
+      </c>
+      <c r="I282" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3 achieves a score of 32%; Kimi K3 achieved ACE on 0/41 samples.</t>
+        </is>
+      </c>
+      <c r="J282" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "Cap%", "value": 32, "unit": "percent", "configuration": "UK AISI／CAISI 2026-07-23初步评估；41个V8漏洞；Kimi部署的选择性评测；Cap与完整ACE分别记录；不继承其他模型的防护关闭设置。"}, {"label": "完整ACE", "value": "0/41", "unit": "ratio", "configuration": "UK AISI／CAISI 2026-07-23初步评估；41个V8漏洞；Kimi部署的选择性评测；Cap与完整ACE分别记录；不继承其他模型的防护关闭设置。"}]</t>
+        </is>
+      </c>
+      <c r="K282" s="10" t="inlineStr">
+        <is>
+          <t>AISI来源32%与GLM来源32.2%是两条独立披露，不擅自提高精度、不覆盖或平均。</t>
+        </is>
+      </c>
+      <c r="L282" s="10" t="inlineStr">
+        <is>
+          <t>UK AISI / CAISI</t>
+        </is>
+      </c>
+      <c r="M282" s="10" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0279</t>
+        </is>
+      </c>
+      <c r="B283" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="C283" s="10" t="inlineStr">
+        <is>
+          <t>The Last Ones (TLO)</t>
+        </is>
+      </c>
+      <c r="D283" s="10" t="inlineStr">
+        <is>
+          <t>已核实数值</t>
+        </is>
+      </c>
+      <c r="E283" s="10" t="inlineStr">
+        <is>
+          <t>平均到达17/32步；10次尝试成功1次</t>
+        </is>
+      </c>
+      <c r="F283" s="10" t="inlineStr"/>
+      <c r="G283" s="10" t="inlineStr">
+        <is>
+          <t>archived_web</t>
+        </is>
+      </c>
+      <c r="H283" s="10" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/aisi-kimi-k3.mhtml Cyber Range: The Last Ones (TLO)</t>
+        </is>
+      </c>
+      <c r="I283" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K3 reached step 17 of this 32-step attack path on average; solved it in 1/10 attempts within the standard 100M token limit.</t>
+        </is>
+      </c>
+      <c r="J283" s="10" t="inlineStr">
+        <is>
+          <t>[{"label": "平均完成步骤", "value": 17, "unit": "count", "configuration": "UK AISI／CAISI 2026-07-23初步评估；The Last Ones为32步企业网络靶场；10次尝试，每次100M token预算；平均进度与成功尝试数分开，不把17步当作成功率。"}, {"label": "端到端成功", "value": "1/10", "unit": "ratio", "configuration": "UK AISI／CAISI 2026-07-23初步评估；The Last Ones为32步企业网络靶场；10次尝试，每次100M token预算；平均进度与成功尝试数分开，不把17步当作成功率。"}]</t>
+        </is>
+      </c>
+      <c r="K283" s="10" t="inlineStr"/>
+      <c r="L283" s="10" t="inlineStr">
+        <is>
+          <t>UK AISI / CAISI</t>
+        </is>
+      </c>
+      <c r="M283" s="10" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0280</t>
+        </is>
+      </c>
+      <c r="B284" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K2.7 Code</t>
+        </is>
+      </c>
+      <c r="C284" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D284" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E284" s="10" t="inlineStr"/>
+      <c r="F284" s="10" t="inlineStr"/>
+      <c r="G284" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H284" s="10" t="inlineStr"/>
+      <c r="I284" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J284" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K284" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="L284" s="10" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="M284" s="10" t="inlineStr">
+        <is>
+          <t>vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0281</t>
+        </is>
+      </c>
+      <c r="B285" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K2.7 Code HighSpeed</t>
+        </is>
+      </c>
+      <c r="C285" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D285" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E285" s="10" t="inlineStr"/>
+      <c r="F285" s="10" t="inlineStr"/>
+      <c r="G285" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H285" s="10" t="inlineStr"/>
+      <c r="I285" s="10" t="inlineStr">
+        <is>
+          <t>同模型服务档位</t>
+        </is>
+      </c>
+      <c r="J285" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K285" s="10" t="inlineStr">
+        <is>
+          <t>同模型服务档位</t>
+        </is>
+      </c>
+      <c r="L285" s="10" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="M285" s="10" t="inlineStr">
+        <is>
+          <t>vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="10" t="inlineStr">
+        <is>
+          <t>CAO-2026-0282</t>
+        </is>
+      </c>
+      <c r="B286" s="10" t="inlineStr">
+        <is>
+          <t>Kimi K2.8 Preview</t>
+        </is>
+      </c>
+      <c r="C286" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="D286" s="10" t="inlineStr">
+        <is>
+          <t>不适用（证据未确认）</t>
+        </is>
+      </c>
+      <c r="E286" s="10" t="inlineStr"/>
+      <c r="F286" s="10" t="inlineStr"/>
+      <c r="G286" s="10" t="inlineStr">
+        <is>
+          <t>不适用</t>
+        </is>
+      </c>
+      <c r="H286" s="10" t="inlineStr"/>
+      <c r="I286" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="J286" s="10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K286" s="10" t="inlineStr">
+        <is>
+          <t>未披露具名项目</t>
+        </is>
+      </c>
+      <c r="L286" s="10" t="inlineStr">
+        <is>
+          <t>Moonshot AI</t>
+        </is>
+      </c>
+      <c r="M286" s="10" t="inlineStr">
+        <is>
+          <t>vendor</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K272"/>
+  <autoFilter ref="A4:M286"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19057,7 +20441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -20364,8 +21748,320 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>kimi-k2-5</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Kimi</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Kimi K2.5</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>1月27日为官方产品演进记录中的模型发布日；2月2日为技术报告提交日，两者分开。</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>1月27日为官方产品演进记录中的模型发布日；2月2日为技术报告提交日，两者分开。</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2602.02276</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-5.pdf</t>
+        </is>
+      </c>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>1月27日为官方产品演进记录中的模型发布日；2月2日为技术报告提交日，两者分开。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>kimi-k2-6</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Kimi</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Kimi K2.6</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>按官方产品演进记录4月20日绘图；原表另列4月21日论坛公告，保留不同事件口径。</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>按官方产品演进记录4月20日绘图；原表另列4月21日论坛公告，保留不同事件口径。</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/moonshotai/Kimi-K2.6</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-6.mhtml</t>
+        </is>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>按官方产品演进记录4月20日绘图；原表另列4月21日论坛公告，保留不同事件口径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>kimi-k2-7-code</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Kimi</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Kimi K2.7 Code</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>官方更新日志确认6月12日发布并开放权重；未确认具名网安成绩，不继承其他Kimi版本。</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>官方更新日志确认6月12日发布并开放权重；未确认具名网安成绩，不继承其他Kimi版本。</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/moonshotai/Kimi-K2.7-Code</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-7-code.mhtml</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>官方更新日志确认6月12日发布并开放权重；未确认具名网安成绩，不继承其他Kimi版本。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>kimi-k2-7-code-highspeed</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Kimi</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Kimi K2.7 Code HighSpeed</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>7月9日为HighSpeed正式上线；6月12日仅预告。同一模型加速档位，不复制独立成绩；共享配置页不是独立模型卡。</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>7月9日为HighSpeed正式上线；6月12日仅预告。同一模型加速档位，不复制独立成绩；共享配置页不是独立模型卡。</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>https://www.kimi.com/en/help/kimi-code/models</t>
+        </is>
+      </c>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-8-preview.mhtml</t>
+        </is>
+      </c>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>7月9日为HighSpeed正式上线；6月12日仅预告。同一模型加速档位，不复制独立成绩；共享配置页不是独立模型卡。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>kimi-k3</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>Kimi</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Kimi K3</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>7月16日为产品／API发布，7月27日为完整权重开放；技术报告、其他厂商比较和独立评测分开保留。</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>7月16日为产品／API发布，7月27日为完整权重开放；技术报告、其他厂商比较和独立评测分开保留。</t>
+        </is>
+      </c>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/MoonshotAI/Kimi-K3/main/k3_tech_report.pdf</t>
+        </is>
+      </c>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k3.pdf</t>
+        </is>
+      </c>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>7月16日为产品／API发布，7月27日为完整权重开放；技术报告、其他厂商比较和独立评测分开保留。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>kimi-k2-8-preview</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>Kimi</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Kimi K2.8 Preview</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>官方更新日志确认9月11日Kimi Code全量上线，仍为预览版；不因共享模型ID或配置页继承K3或K2.7成绩。</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>官方更新日志确认9月11日Kimi Code全量上线，仍为预览版；不因共享模型ID或配置页继承K3或K2.7成绩。</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>https://www.kimi.com/en/help/kimi-code/models</t>
+        </is>
+      </c>
+      <c r="I32" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-8-preview.mhtml</t>
+        </is>
+      </c>
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>官方更新日志确认9月11日Kimi Code全量上线，仍为预览版；不因共享模型ID或配置页继承K3或K2.7成绩。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J26"/>
+  <autoFilter ref="A1:J32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20376,7 +22072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -21499,8 +23195,308 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/aisi-kimi-k3.mhtml</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>9e0e6add23c69c6a7d577c1d7e7609d6431f28335a9f6c065497da7dae6ec55e</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>https://www.aisi.gov.uk/blog/preliminary-assessment-of-kimi-k3s-cyber-capabilities</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T11:57:07+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-code-changelog.mhtml</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>0c0034796e3950f134d6d9dd6dd86a16a826500a3c1e7a9cff05d34e1fd04f6b</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>https://www.kimi.com/code/docs/en/kimi-code/whats-new.html</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T11:57:08+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-5.pdf</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>官方原始 PDF</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>889025c0fcbacb8b049aacd5b21f6c902a236eb28dec7aa51e6852ca39ec5417</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2602.02276</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-6.mhtml</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>b75c00c64576896c669a1335d79cb234d9e16f945b5ca739beae857346fc585c</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/moonshotai/Kimi-K2.6</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T11:57:04+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-7-code.mhtml</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>a4e61fd94b6408158c3fe63d9df56dd3b929b03382f5156bcc209d83b3631d60</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/moonshotai/Kimi-K2.7-Code</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T11:57:04+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k2-8-preview.mhtml</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>a8f69993ce58925e7ac6c686418554d0678d0d48793fa665237c0ba875049495</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>https://www.kimi.com/en/help/kimi-code/models</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T11:57:04+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/kimi-k3.pdf</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>官方原始 PDF</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>86fb82a63ced501f0c3f4f404c0c6fa88a7a6cfac17aae81fd1a8f455998067c</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/MoonshotAI/Kimi-K3/main/k3_tech_report.pdf</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/release-history.html</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>ceb8d3a8e2a58163a0c16094f5bb25490656db592d4b3ad4e470b13b8297fc58</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>https://www.kimi.ai/help/agent/agent-overview</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/vals-cyberbench-v1-1.mhtml</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>0640c02419c8893446e52f63b6a3ed8d8eb214ce42902593c425afd559b2fcad</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>https://www.vals.ai/benchmarks/cyber</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T11:57:11+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>sources/vendors/Moonshot/vals-cyberbench-v1.mhtml</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>MHTML</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>c5b56da7d148da7cacc78535f1f4f5dd6de7e58a7fdd8c195f5bbf0197285d81</t>
+        </is>
+      </c>
+      <c r="E47" s="12" t="inlineStr">
+        <is>
+          <t>https://www.vals.ai/benchmarks/cyber-v1</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18T11:57:08+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F37"/>
+  <autoFilter ref="A1:F47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>